<commit_message>
Daily attendance update - 2026-09-09
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FECA2539-C736-45B6-A4F9-4C509092C101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66A6409C-3C53-4877-B56B-FC99B6DBCFF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="17" activeTab="19" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="17" activeTab="20" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3176" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3212" uniqueCount="33">
   <si>
     <t>Person</t>
   </si>
@@ -11102,7 +11102,7 @@
     <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
@@ -11341,14 +11341,26 @@
       <c r="H3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="I3" s="10"/>
+      <c r="I3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="10"/>
+      <c r="L3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="Q3" s="7"/>
       <c r="R3" s="7"/>
       <c r="S3" s="10"/>
@@ -11394,14 +11406,26 @@
       <c r="H4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="I4" s="10"/>
+      <c r="I4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J4" s="7"/>
       <c r="K4" s="7"/>
-      <c r="L4" s="10"/>
-      <c r="M4" s="10"/>
-      <c r="N4" s="10"/>
-      <c r="O4" s="10"/>
-      <c r="P4" s="10"/>
+      <c r="L4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="P4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="Q4" s="7"/>
       <c r="R4" s="7"/>
       <c r="S4" s="10"/>
@@ -11447,14 +11471,26 @@
       <c r="H5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="10"/>
+      <c r="I5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J5" s="7"/>
       <c r="K5" s="7"/>
-      <c r="L5" s="10"/>
-      <c r="M5" s="10"/>
-      <c r="N5" s="10"/>
-      <c r="O5" s="10"/>
-      <c r="P5" s="10"/>
+      <c r="L5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="Q5" s="7"/>
       <c r="R5" s="7"/>
       <c r="S5" s="10"/>
@@ -11500,14 +11536,26 @@
       <c r="H6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="10"/>
+      <c r="I6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J6" s="7"/>
       <c r="K6" s="7"/>
-      <c r="L6" s="10"/>
-      <c r="M6" s="10"/>
-      <c r="N6" s="10"/>
-      <c r="O6" s="10"/>
-      <c r="P6" s="10"/>
+      <c r="L6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="Q6" s="7"/>
       <c r="R6" s="7"/>
       <c r="S6" s="10"/>
@@ -11553,14 +11601,26 @@
       <c r="H7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="10"/>
+      <c r="I7" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
-      <c r="L7" s="10"/>
-      <c r="M7" s="10"/>
-      <c r="N7" s="10"/>
-      <c r="O7" s="10"/>
-      <c r="P7" s="10"/>
+      <c r="L7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="P7" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="Q7" s="7"/>
       <c r="R7" s="7"/>
       <c r="S7" s="10"/>
@@ -11606,14 +11666,26 @@
       <c r="H8" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="I8" s="10"/>
+      <c r="I8" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10"/>
-      <c r="O8" s="10"/>
-      <c r="P8" s="10"/>
+      <c r="L8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="N8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="O8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="P8" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="Q8" s="7"/>
       <c r="R8" s="7"/>
       <c r="S8" s="10"/>
@@ -11651,11 +11723,11 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(H5:AI5,"WFH")</f>
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
@@ -11664,11 +11736,11 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F7:AI7,"WFO")</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(H7:AI7,"WFH")</f>
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
@@ -11677,11 +11749,11 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F8:AI8,"WFO")</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(H8:AI8,"WFH")</f>
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-09-15
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66A6409C-3C53-4877-B56B-FC99B6DBCFF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E868B83F-BD3B-4243-8153-3BDEB81ECC15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="17" activeTab="20" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3212" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3225" uniqueCount="33">
   <si>
     <t>Person</t>
   </si>
@@ -11363,8 +11363,12 @@
       </c>
       <c r="Q3" s="7"/>
       <c r="R3" s="7"/>
-      <c r="S3" s="10"/>
-      <c r="T3" s="10"/>
+      <c r="S3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="T3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="U3" s="10"/>
       <c r="V3" s="10"/>
       <c r="W3" s="10"/>
@@ -11428,8 +11432,12 @@
       </c>
       <c r="Q4" s="7"/>
       <c r="R4" s="7"/>
-      <c r="S4" s="10"/>
-      <c r="T4" s="10"/>
+      <c r="S4" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="T4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="U4" s="10"/>
       <c r="V4" s="10"/>
       <c r="W4" s="10"/>
@@ -11493,8 +11501,12 @@
       </c>
       <c r="Q5" s="7"/>
       <c r="R5" s="7"/>
-      <c r="S5" s="10"/>
-      <c r="T5" s="10"/>
+      <c r="S5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="T5" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="U5" s="10"/>
       <c r="V5" s="10"/>
       <c r="W5" s="10"/>
@@ -11558,8 +11570,12 @@
       </c>
       <c r="Q6" s="7"/>
       <c r="R6" s="7"/>
-      <c r="S6" s="10"/>
-      <c r="T6" s="10"/>
+      <c r="S6" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="T6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="U6" s="10"/>
       <c r="V6" s="10"/>
       <c r="W6" s="10"/>
@@ -11623,8 +11639,12 @@
       </c>
       <c r="Q7" s="7"/>
       <c r="R7" s="7"/>
-      <c r="S7" s="10"/>
-      <c r="T7" s="10"/>
+      <c r="S7" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="T7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="U7" s="10"/>
       <c r="V7" s="10"/>
       <c r="W7" s="10"/>
@@ -11688,9 +11708,15 @@
       </c>
       <c r="Q8" s="7"/>
       <c r="R8" s="7"/>
-      <c r="S8" s="10"/>
-      <c r="T8" s="10"/>
-      <c r="U8" s="10"/>
+      <c r="S8" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="T8" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="U8" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="V8" s="10"/>
       <c r="W8" s="10"/>
       <c r="X8" s="7"/>
@@ -11736,7 +11762,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F7:AI7,"WFO")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(H7:AI7,"WFH")</f>

</xml_diff>

<commit_message>
Daily attendance update - 2026-09-21
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E868B83F-BD3B-4243-8153-3BDEB81ECC15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B37BDD2-660F-4556-A2A3-90C9E39564F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="17" activeTab="20" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3225" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3248" uniqueCount="33">
   <si>
     <t>Person</t>
   </si>
@@ -11369,12 +11369,20 @@
       <c r="T3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="U3" s="10"/>
-      <c r="V3" s="10"/>
-      <c r="W3" s="10"/>
+      <c r="U3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="X3" s="7"/>
       <c r="Y3" s="7"/>
-      <c r="Z3" s="10"/>
+      <c r="Z3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AA3" s="10"/>
       <c r="AB3" s="10"/>
       <c r="AC3" s="10"/>
@@ -11438,12 +11446,20 @@
       <c r="T4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="U4" s="10"/>
-      <c r="V4" s="10"/>
-      <c r="W4" s="10"/>
+      <c r="U4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="X4" s="7"/>
       <c r="Y4" s="7"/>
-      <c r="Z4" s="10"/>
+      <c r="Z4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AA4" s="10"/>
       <c r="AB4" s="10"/>
       <c r="AC4" s="10"/>
@@ -11507,12 +11523,20 @@
       <c r="T5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="U5" s="10"/>
-      <c r="V5" s="10"/>
-      <c r="W5" s="10"/>
+      <c r="U5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="V5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="W5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="X5" s="7"/>
       <c r="Y5" s="7"/>
-      <c r="Z5" s="10"/>
+      <c r="Z5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AA5" s="10"/>
       <c r="AB5" s="10"/>
       <c r="AC5" s="10"/>
@@ -11576,12 +11600,20 @@
       <c r="T6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="U6" s="10"/>
-      <c r="V6" s="10"/>
-      <c r="W6" s="10"/>
+      <c r="U6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="V6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="W6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="X6" s="7"/>
       <c r="Y6" s="7"/>
-      <c r="Z6" s="10"/>
+      <c r="Z6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AA6" s="10"/>
       <c r="AB6" s="10"/>
       <c r="AC6" s="10"/>
@@ -11645,12 +11677,20 @@
       <c r="T7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="U7" s="10"/>
-      <c r="V7" s="10"/>
-      <c r="W7" s="10"/>
+      <c r="U7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="V7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="W7" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="X7" s="7"/>
       <c r="Y7" s="7"/>
-      <c r="Z7" s="10"/>
+      <c r="Z7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AA7" s="10"/>
       <c r="AB7" s="10"/>
       <c r="AC7" s="10"/>
@@ -11717,11 +11757,17 @@
       <c r="U8" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="V8" s="10"/>
-      <c r="W8" s="10"/>
+      <c r="V8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="W8" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="X8" s="7"/>
       <c r="Y8" s="7"/>
-      <c r="Z8" s="10"/>
+      <c r="Z8" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AA8" s="10"/>
       <c r="AB8" s="10"/>
       <c r="AC8" s="10"/>
@@ -11749,11 +11795,11 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(H5:AI5,"WFH")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
@@ -11762,11 +11808,11 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F7:AI7,"WFO")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(H7:AI7,"WFH")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
@@ -11775,11 +11821,11 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F8:AI8,"WFO")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(H8:AI8,"WFH")</f>
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-09-24
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B37BDD2-660F-4556-A2A3-90C9E39564F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41026C79-9923-4E52-A48D-554D0A49A67C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="17" activeTab="20" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="17" activeTab="20" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3248" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3272" uniqueCount="33">
   <si>
     <t>Person</t>
   </si>
@@ -11383,10 +11383,18 @@
       <c r="Z3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AA3" s="10"/>
-      <c r="AB3" s="10"/>
-      <c r="AC3" s="10"/>
-      <c r="AD3" s="10"/>
+      <c r="AA3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AE3" s="7"/>
       <c r="AF3" s="7"/>
       <c r="AG3" s="10"/>
@@ -11460,10 +11468,18 @@
       <c r="Z4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AA4" s="10"/>
-      <c r="AB4" s="10"/>
-      <c r="AC4" s="10"/>
-      <c r="AD4" s="10"/>
+      <c r="AA4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AE4" s="7"/>
       <c r="AF4" s="7"/>
       <c r="AG4" s="10"/>
@@ -11537,10 +11553,18 @@
       <c r="Z5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AA5" s="10"/>
-      <c r="AB5" s="10"/>
-      <c r="AC5" s="10"/>
-      <c r="AD5" s="10"/>
+      <c r="AA5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AE5" s="7"/>
       <c r="AF5" s="7"/>
       <c r="AG5" s="10"/>
@@ -11614,10 +11638,18 @@
       <c r="Z6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AA6" s="10"/>
-      <c r="AB6" s="10"/>
-      <c r="AC6" s="10"/>
-      <c r="AD6" s="10"/>
+      <c r="AA6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AE6" s="7"/>
       <c r="AF6" s="7"/>
       <c r="AG6" s="10"/>
@@ -11691,10 +11723,18 @@
       <c r="Z7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AA7" s="10"/>
-      <c r="AB7" s="10"/>
-      <c r="AC7" s="10"/>
-      <c r="AD7" s="10"/>
+      <c r="AA7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD7" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
       <c r="AG7" s="10"/>
@@ -11768,10 +11808,18 @@
       <c r="Z8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AA8" s="10"/>
-      <c r="AB8" s="10"/>
-      <c r="AC8" s="10"/>
-      <c r="AD8" s="10"/>
+      <c r="AA8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD8" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AE8" s="7"/>
       <c r="AF8" s="7"/>
       <c r="AG8" s="10"/>
@@ -11795,11 +11843,11 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(H5:AI5,"WFH")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
@@ -11808,11 +11856,11 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F7:AI7,"WFO")</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(H7:AI7,"WFH")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
@@ -11821,11 +11869,11 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F8:AI8,"WFO")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(H8:AI8,"WFH")</f>
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-09-29
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41026C79-9923-4E52-A48D-554D0A49A67C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9015065-EF3B-4A13-B136-4AAF38DCFE10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="17" activeTab="20" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" firstSheet="17" activeTab="20" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3272" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3290" uniqueCount="33">
   <si>
     <t>Person</t>
   </si>
@@ -230,7 +230,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -267,12 +267,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -345,7 +339,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -362,7 +356,6 @@
     <xf numFmtId="164" fontId="3" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1293,19 +1286,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -1403,11 +1396,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>9</v>
       </c>
@@ -2088,19 +2081,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -2198,11 +2191,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>9</v>
       </c>
@@ -2821,19 +2814,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -2928,11 +2921,11 @@
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
@@ -3520,19 +3513,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -3630,11 +3623,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
@@ -4254,19 +4247,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -4364,11 +4357,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>10</v>
       </c>
@@ -4979,19 +4972,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -5080,11 +5073,11 @@
       </c>
     </row>
     <row r="2" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>6</v>
       </c>
@@ -5656,19 +5649,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -5766,11 +5759,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>6</v>
       </c>
@@ -6382,19 +6375,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -6489,11 +6482,11 @@
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>9</v>
       </c>
@@ -7099,19 +7092,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -7209,11 +7202,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>11</v>
       </c>
@@ -7817,19 +7810,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -7924,11 +7917,11 @@
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
@@ -8586,19 +8579,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -8696,11 +8689,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>9</v>
       </c>
@@ -9530,19 +9523,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -9631,11 +9624,11 @@
       </c>
     </row>
     <row r="2" spans="1:33" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
@@ -10264,19 +10257,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -10374,11 +10367,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
@@ -11113,19 +11106,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -11220,11 +11213,11 @@
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>8</v>
       </c>
@@ -11397,9 +11390,15 @@
       </c>
       <c r="AE3" s="7"/>
       <c r="AF3" s="7"/>
-      <c r="AG3" s="10"/>
-      <c r="AH3" s="10"/>
-      <c r="AI3" s="10"/>
+      <c r="AG3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI3" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -11482,9 +11481,15 @@
       </c>
       <c r="AE4" s="7"/>
       <c r="AF4" s="7"/>
-      <c r="AG4" s="10"/>
-      <c r="AH4" s="10"/>
-      <c r="AI4" s="10"/>
+      <c r="AG4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI4" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -11567,9 +11572,15 @@
       </c>
       <c r="AE5" s="7"/>
       <c r="AF5" s="7"/>
-      <c r="AG5" s="10"/>
-      <c r="AH5" s="10"/>
-      <c r="AI5" s="10"/>
+      <c r="AG5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AH5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI5" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -11652,9 +11663,15 @@
       </c>
       <c r="AE6" s="7"/>
       <c r="AF6" s="7"/>
-      <c r="AG6" s="10"/>
-      <c r="AH6" s="10"/>
-      <c r="AI6" s="10"/>
+      <c r="AG6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="AH6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI6" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
@@ -11737,9 +11754,15 @@
       </c>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
-      <c r="AG7" s="10"/>
-      <c r="AH7" s="10"/>
-      <c r="AI7" s="10"/>
+      <c r="AG7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AI7" s="6" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="8" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
@@ -11822,9 +11845,15 @@
       </c>
       <c r="AE8" s="7"/>
       <c r="AF8" s="7"/>
-      <c r="AG8" s="10"/>
-      <c r="AH8" s="10"/>
-      <c r="AI8" s="10"/>
+      <c r="AG8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI8" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
@@ -11843,11 +11872,11 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(H5:AI5,"WFH")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
@@ -11856,7 +11885,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F7:AI7,"WFO")</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(H7:AI7,"WFH")</f>
@@ -11869,11 +11898,11 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F8:AI8,"WFO")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(H8:AI8,"WFH")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -11926,19 +11955,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -12036,11 +12065,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>5</v>
       </c>
@@ -12221,7 +12250,7 @@
       </c>
       <c r="AH3" s="2"/>
       <c r="AI3" s="2"/>
-      <c r="AJ3" s="13" t="s">
+      <c r="AJ3" s="12" t="s">
         <v>25</v>
       </c>
     </row>
@@ -12311,7 +12340,7 @@
       </c>
       <c r="AH4" s="2"/>
       <c r="AI4" s="2"/>
-      <c r="AJ4" s="14"/>
+      <c r="AJ4" s="13"/>
     </row>
     <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
@@ -12399,7 +12428,7 @@
       </c>
       <c r="AH5" s="2"/>
       <c r="AI5" s="2"/>
-      <c r="AJ5" s="14"/>
+      <c r="AJ5" s="13"/>
     </row>
     <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
@@ -12487,7 +12516,7 @@
       </c>
       <c r="AH6" s="2"/>
       <c r="AI6" s="2"/>
-      <c r="AJ6" s="14"/>
+      <c r="AJ6" s="13"/>
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
@@ -12525,7 +12554,7 @@
       <c r="AG7" s="2"/>
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
-      <c r="AJ7" s="15"/>
+      <c r="AJ7" s="14"/>
     </row>
     <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
@@ -12638,19 +12667,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -12745,11 +12774,11 @@
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>8</v>
       </c>
@@ -13353,19 +13382,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -13463,11 +13492,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>10</v>
       </c>
@@ -14068,19 +14097,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -14175,11 +14204,11 @@
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>6</v>
       </c>
@@ -14765,19 +14794,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -14875,11 +14904,11 @@
       </c>
     </row>
     <row r="2" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>8</v>
       </c>
@@ -15489,19 +15518,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -15600,11 +15629,11 @@
       <c r="AK1" s="1"/>
     </row>
     <row r="2" spans="1:37" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>11</v>
       </c>
@@ -16200,19 +16229,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="1">
@@ -16307,11 +16336,11 @@
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
       <c r="F2" s="1" t="s">
         <v>7</v>
       </c>

</xml_diff>

<commit_message>
Daily attendance update - 2026-10-08
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9015065-EF3B-4A13-B136-4AAF38DCFE10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2B4E08A-320F-48DF-ACBB-2C055B73DA32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" firstSheet="17" activeTab="20" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="18" activeTab="21" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -34,6 +34,7 @@
     <sheet name="UV-WMS Admin July 2026" sheetId="19" r:id="rId19"/>
     <sheet name="UV-WMS Admin Aug 2026" sheetId="20" r:id="rId20"/>
     <sheet name="UV-WMS Admin Sep 2026" sheetId="21" r:id="rId21"/>
+    <sheet name="UV-WMS Admin Oct 2026" sheetId="22" r:id="rId22"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -56,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3290" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3392" uniqueCount="33">
   <si>
     <t>Person</t>
   </si>
@@ -379,7 +380,37 @@
     <cellStyle name="Neutral" xfId="4" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="55">
+  <dxfs count="58">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -2777,13 +2808,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="35" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="38" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="37" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="36" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3475,13 +3506,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="32" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="35" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="34" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="33" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4209,13 +4240,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="31" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="30" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4935,13 +4966,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="27" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5611,13 +5642,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6337,13 +6368,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="23" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="22" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7052,13 +7083,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="19" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7772,13 +7803,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8541,13 +8572,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9481,13 +9512,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B14:B17">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11066,13 +11097,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B13:B15">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11903,6 +11934,676 @@
       <c r="C15" s="2">
         <f>COUNTIF(H8:AI8,"WFH")</f>
         <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+  </mergeCells>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <conditionalFormatting sqref="B13:B15">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
+      <formula>11</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+      <formula>12</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+      <formula>12</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A2B8991-FECB-4DED-BEB7-2ACC94684DF5}">
+  <dimension ref="A1:AJ15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="12.85546875" customWidth="1"/>
+    <col min="8" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1">
+        <v>46296</v>
+      </c>
+      <c r="G1" s="1">
+        <v>46297</v>
+      </c>
+      <c r="H1" s="1">
+        <v>46298</v>
+      </c>
+      <c r="I1" s="1">
+        <v>46299</v>
+      </c>
+      <c r="J1" s="1">
+        <v>46300</v>
+      </c>
+      <c r="K1" s="1">
+        <v>46301</v>
+      </c>
+      <c r="L1" s="1">
+        <v>46302</v>
+      </c>
+      <c r="M1" s="1">
+        <v>46303</v>
+      </c>
+      <c r="N1" s="1">
+        <v>46304</v>
+      </c>
+      <c r="O1" s="1">
+        <v>46305</v>
+      </c>
+      <c r="P1" s="1">
+        <v>46306</v>
+      </c>
+      <c r="Q1" s="1">
+        <v>46307</v>
+      </c>
+      <c r="R1" s="1">
+        <v>46308</v>
+      </c>
+      <c r="S1" s="1">
+        <v>46309</v>
+      </c>
+      <c r="T1" s="1">
+        <v>46310</v>
+      </c>
+      <c r="U1" s="1">
+        <v>46311</v>
+      </c>
+      <c r="V1" s="1">
+        <v>46312</v>
+      </c>
+      <c r="W1" s="1">
+        <v>46313</v>
+      </c>
+      <c r="X1" s="1">
+        <v>46314</v>
+      </c>
+      <c r="Y1" s="1">
+        <v>46315</v>
+      </c>
+      <c r="Z1" s="1">
+        <v>46316</v>
+      </c>
+      <c r="AA1" s="1">
+        <v>46317</v>
+      </c>
+      <c r="AB1" s="1">
+        <v>46318</v>
+      </c>
+      <c r="AC1" s="1">
+        <v>46319</v>
+      </c>
+      <c r="AD1" s="1">
+        <v>46320</v>
+      </c>
+      <c r="AE1" s="1">
+        <v>46321</v>
+      </c>
+      <c r="AF1" s="1">
+        <v>46322</v>
+      </c>
+      <c r="AG1" s="1">
+        <v>46323</v>
+      </c>
+      <c r="AH1" s="1">
+        <v>46324</v>
+      </c>
+      <c r="AI1" s="1">
+        <v>46325</v>
+      </c>
+      <c r="AJ1" s="1">
+        <v>46326</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AB2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="AD2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="AE2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="AF2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AG2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="AH2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AI2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="AJ2" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="2">
+        <v>51690</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N3" s="2"/>
+      <c r="O3" s="7"/>
+      <c r="P3" s="7"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
+      <c r="U3" s="2"/>
+      <c r="V3" s="7"/>
+      <c r="W3" s="7"/>
+      <c r="X3" s="2"/>
+      <c r="Y3" s="2"/>
+      <c r="Z3" s="2"/>
+      <c r="AA3" s="2"/>
+      <c r="AB3" s="2"/>
+      <c r="AC3" s="7"/>
+      <c r="AD3" s="7"/>
+      <c r="AE3" s="2"/>
+      <c r="AF3" s="2"/>
+      <c r="AG3" s="2"/>
+      <c r="AH3" s="2"/>
+      <c r="AI3" s="2"/>
+      <c r="AJ3" s="7"/>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="2">
+        <v>35898</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N4" s="2"/>
+      <c r="O4" s="7"/>
+      <c r="P4" s="7"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="2"/>
+      <c r="T4" s="2"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="7"/>
+      <c r="W4" s="7"/>
+      <c r="X4" s="2"/>
+      <c r="Y4" s="2"/>
+      <c r="Z4" s="2"/>
+      <c r="AA4" s="2"/>
+      <c r="AB4" s="2"/>
+      <c r="AC4" s="7"/>
+      <c r="AD4" s="7"/>
+      <c r="AE4" s="2"/>
+      <c r="AF4" s="2"/>
+      <c r="AG4" s="2"/>
+      <c r="AH4" s="2"/>
+      <c r="AI4" s="2"/>
+      <c r="AJ4" s="7"/>
+    </row>
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="2">
+        <v>35898</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="N5" s="2"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="2"/>
+      <c r="T5" s="2"/>
+      <c r="U5" s="2"/>
+      <c r="V5" s="7"/>
+      <c r="W5" s="7"/>
+      <c r="X5" s="2"/>
+      <c r="Y5" s="2"/>
+      <c r="Z5" s="2"/>
+      <c r="AA5" s="2"/>
+      <c r="AB5" s="2"/>
+      <c r="AC5" s="7"/>
+      <c r="AD5" s="7"/>
+      <c r="AE5" s="2"/>
+      <c r="AF5" s="2"/>
+      <c r="AG5" s="2"/>
+      <c r="AH5" s="2"/>
+      <c r="AI5" s="2"/>
+      <c r="AJ5" s="7"/>
+    </row>
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="2">
+        <v>52370</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N6" s="2"/>
+      <c r="O6" s="7"/>
+      <c r="P6" s="7"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
+      <c r="S6" s="2"/>
+      <c r="T6" s="2"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="7"/>
+      <c r="W6" s="7"/>
+      <c r="X6" s="2"/>
+      <c r="Y6" s="2"/>
+      <c r="Z6" s="2"/>
+      <c r="AA6" s="2"/>
+      <c r="AB6" s="2"/>
+      <c r="AC6" s="7"/>
+      <c r="AD6" s="7"/>
+      <c r="AE6" s="2"/>
+      <c r="AF6" s="2"/>
+      <c r="AG6" s="2"/>
+      <c r="AH6" s="2"/>
+      <c r="AI6" s="2"/>
+      <c r="AJ6" s="7"/>
+    </row>
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="2">
+        <v>33548</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N7" s="2"/>
+      <c r="O7" s="7"/>
+      <c r="P7" s="7"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="2"/>
+      <c r="T7" s="2"/>
+      <c r="U7" s="2"/>
+      <c r="V7" s="7"/>
+      <c r="W7" s="7"/>
+      <c r="X7" s="2"/>
+      <c r="Y7" s="2"/>
+      <c r="Z7" s="2"/>
+      <c r="AA7" s="2"/>
+      <c r="AB7" s="2"/>
+      <c r="AC7" s="7"/>
+      <c r="AD7" s="7"/>
+      <c r="AE7" s="2"/>
+      <c r="AF7" s="2"/>
+      <c r="AG7" s="2"/>
+      <c r="AH7" s="2"/>
+      <c r="AI7" s="2"/>
+      <c r="AJ7" s="7"/>
+    </row>
+    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2">
+        <v>44429</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N8" s="2"/>
+      <c r="O8" s="7"/>
+      <c r="P8" s="7"/>
+      <c r="Q8" s="2"/>
+      <c r="R8" s="2"/>
+      <c r="S8" s="2"/>
+      <c r="T8" s="2"/>
+      <c r="U8" s="2"/>
+      <c r="V8" s="7"/>
+      <c r="W8" s="7"/>
+      <c r="X8" s="2"/>
+      <c r="Y8" s="2"/>
+      <c r="Z8" s="2"/>
+      <c r="AA8" s="2"/>
+      <c r="AB8" s="2"/>
+      <c r="AC8" s="7"/>
+      <c r="AD8" s="7"/>
+      <c r="AE8" s="2"/>
+      <c r="AF8" s="2"/>
+      <c r="AG8" s="2"/>
+      <c r="AH8" s="2"/>
+      <c r="AI8" s="2"/>
+      <c r="AJ8" s="7"/>
+    </row>
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A12" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <f>COUNTIF(F5:AI5,"WFO")</f>
+        <v>3</v>
+      </c>
+      <c r="C13" s="2">
+        <f>COUNTIF(H5:AI5,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="2">
+        <f>COUNTIF(F7:AI7,"WFO")</f>
+        <v>3</v>
+      </c>
+      <c r="C14" s="2">
+        <f>COUNTIF(H7:AI7,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="2">
+        <f>COUNTIF(F8:AI8,"WFO")</f>
+        <v>3</v>
+      </c>
+      <c r="C15" s="2">
+        <f>COUNTIF(H8:AI8,"WFH")</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -12629,10 +13330,10 @@
     <mergeCell ref="E1:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="B10:B13">
-    <cfRule type="cellIs" dxfId="54" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="57" priority="1" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="53" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="56" priority="2" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13344,10 +14045,10 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B11:B14">
-    <cfRule type="cellIs" dxfId="52" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="55" priority="1" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="54" priority="2" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14069,15 +14770,15 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B11:B14">
-    <cfRule type="cellIs" dxfId="50" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="53" priority="2" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="52" priority="4" operator="lessThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:B14">
-    <cfRule type="cellIs" dxfId="48" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="51" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14766,13 +15467,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="47" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="50" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="49" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="48" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15489,13 +16190,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="44" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="47" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="46" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="45" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16199,13 +16900,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="41" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="44" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="43" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="42" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16906,13 +17607,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="38" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="41" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="40" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="39" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Daily attendance update - 2026-10-13
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2B4E08A-320F-48DF-ACBB-2C055B73DA32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D2CC655-02B6-43E7-94CC-13D33AC75A2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="18" activeTab="21" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="20" activeTab="21" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -35,6 +35,8 @@
     <sheet name="UV-WMS Admin Aug 2026" sheetId="20" r:id="rId20"/>
     <sheet name="UV-WMS Admin Sep 2026" sheetId="21" r:id="rId21"/>
     <sheet name="UV-WMS Admin Oct 2026" sheetId="22" r:id="rId22"/>
+    <sheet name="UV-WMS Admin Nov 2026" sheetId="23" r:id="rId23"/>
+    <sheet name="UV-WMS Admin Dec 2026" sheetId="25" r:id="rId24"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -57,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3392" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3548" uniqueCount="33">
   <si>
     <t>Person</t>
   </si>
@@ -380,7 +382,67 @@
     <cellStyle name="Neutral" xfId="4" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="58">
+  <dxfs count="64">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -2808,13 +2870,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="38" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="44" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="43" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="42" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3506,13 +3568,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="35" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="41" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="40" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="39" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4240,13 +4302,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="32" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="38" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="37" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="36" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4966,13 +5028,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="35" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="34" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="33" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5642,13 +5704,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="26" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="31" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="30" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6368,13 +6430,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="23" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="27" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7083,13 +7145,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="25" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7803,13 +7865,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="23" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="22" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8572,13 +8634,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="20" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="19" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9512,13 +9574,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B14:B17">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11097,13 +11159,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B13:B15">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11946,13 +12008,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B13:B15">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11973,12 +12035,13 @@
     <col min="6" max="7" width="12.85546875" customWidth="1"/>
     <col min="8" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
@@ -12232,11 +12295,17 @@
       <c r="M3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="N3" s="2"/>
+      <c r="N3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="O3" s="7"/>
       <c r="P3" s="7"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
+      <c r="Q3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="S3" s="2"/>
       <c r="T3" s="2"/>
       <c r="U3" s="2"/>
@@ -12292,14 +12361,26 @@
       <c r="M4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="N4" s="2"/>
+      <c r="N4" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="O4" s="7"/>
       <c r="P4" s="7"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="2"/>
-      <c r="T4" s="2"/>
-      <c r="U4" s="2"/>
+      <c r="Q4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="R4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="S4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="T4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="U4" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="V4" s="7"/>
       <c r="W4" s="7"/>
       <c r="X4" s="2"/>
@@ -12352,11 +12433,17 @@
       <c r="M5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="N5" s="2"/>
+      <c r="N5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="O5" s="7"/>
       <c r="P5" s="7"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
+      <c r="Q5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="R5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="S5" s="2"/>
       <c r="T5" s="2"/>
       <c r="U5" s="2"/>
@@ -12409,14 +12496,20 @@
       <c r="L6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="M6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="N6" s="2"/>
+      <c r="M6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="O6" s="7"/>
       <c r="P6" s="7"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
+      <c r="Q6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="R6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="S6" s="2"/>
       <c r="T6" s="2"/>
       <c r="U6" s="2"/>
@@ -12472,11 +12565,17 @@
       <c r="M7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="N7" s="2"/>
+      <c r="N7" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
-      <c r="Q7" s="2"/>
-      <c r="R7" s="2"/>
+      <c r="Q7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="R7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="S7" s="2"/>
       <c r="T7" s="2"/>
       <c r="U7" s="2"/>
@@ -12532,11 +12631,17 @@
       <c r="M8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="N8" s="2"/>
+      <c r="N8" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
+      <c r="Q8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="R8" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="S8" s="2"/>
       <c r="T8" s="2"/>
       <c r="U8" s="2"/>
@@ -12573,20 +12678,1205 @@
       </c>
       <c r="B13" s="2">
         <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>3</v>
+        <v>5</v>
+      </c>
+      <c r="C13" s="2">
+        <f>COUNTIF(H5:AI5,"WFH")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="2">
+        <f>COUNTIF(F7:AI7,"WFO")</f>
+        <v>5</v>
+      </c>
+      <c r="C14" s="2">
+        <f>COUNTIF(H7:AI7,"WFH")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="2">
+        <f>COUNTIF(F8:AI8,"WFO")</f>
+        <v>5</v>
+      </c>
+      <c r="C15" s="2">
+        <f>COUNTIF(H8:AI8,"WFH")</f>
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+  </mergeCells>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <conditionalFormatting sqref="B13:B15">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
+      <formula>11</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
+      <formula>12</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
+      <formula>12</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4E8A644-1993-49C0-933B-42395C786DC4}">
+  <dimension ref="A1:AI15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="22" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="24" max="29" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="31" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1">
+        <v>46327</v>
+      </c>
+      <c r="G1" s="1">
+        <v>46328</v>
+      </c>
+      <c r="H1" s="1">
+        <v>46329</v>
+      </c>
+      <c r="I1" s="1">
+        <v>46330</v>
+      </c>
+      <c r="J1" s="1">
+        <v>46331</v>
+      </c>
+      <c r="K1" s="1">
+        <v>46332</v>
+      </c>
+      <c r="L1" s="1">
+        <v>46333</v>
+      </c>
+      <c r="M1" s="1">
+        <v>46334</v>
+      </c>
+      <c r="N1" s="1">
+        <v>46335</v>
+      </c>
+      <c r="O1" s="1">
+        <v>46336</v>
+      </c>
+      <c r="P1" s="1">
+        <v>46337</v>
+      </c>
+      <c r="Q1" s="1">
+        <v>46338</v>
+      </c>
+      <c r="R1" s="1">
+        <v>46339</v>
+      </c>
+      <c r="S1" s="1">
+        <v>46340</v>
+      </c>
+      <c r="T1" s="1">
+        <v>46341</v>
+      </c>
+      <c r="U1" s="1">
+        <v>46342</v>
+      </c>
+      <c r="V1" s="1">
+        <v>46343</v>
+      </c>
+      <c r="W1" s="1">
+        <v>46344</v>
+      </c>
+      <c r="X1" s="1">
+        <v>46345</v>
+      </c>
+      <c r="Y1" s="1">
+        <v>46346</v>
+      </c>
+      <c r="Z1" s="1">
+        <v>46347</v>
+      </c>
+      <c r="AA1" s="1">
+        <v>46348</v>
+      </c>
+      <c r="AB1" s="1">
+        <v>46349</v>
+      </c>
+      <c r="AC1" s="1">
+        <v>46350</v>
+      </c>
+      <c r="AD1" s="1">
+        <v>46351</v>
+      </c>
+      <c r="AE1" s="1">
+        <v>46352</v>
+      </c>
+      <c r="AF1" s="1">
+        <v>46353</v>
+      </c>
+      <c r="AG1" s="1">
+        <v>46354</v>
+      </c>
+      <c r="AH1" s="1">
+        <v>46355</v>
+      </c>
+      <c r="AI1" s="1">
+        <v>46356</v>
+      </c>
+    </row>
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="AB2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="AC2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AD2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="AE2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AF2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="AG2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="AH2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI2" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="2">
+        <v>51690</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="7"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="7"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="7"/>
+      <c r="T3" s="7"/>
+      <c r="U3" s="2"/>
+      <c r="V3" s="2"/>
+      <c r="W3" s="2"/>
+      <c r="X3" s="2"/>
+      <c r="Y3" s="2"/>
+      <c r="Z3" s="7"/>
+      <c r="AA3" s="7"/>
+      <c r="AB3" s="2"/>
+      <c r="AC3" s="2"/>
+      <c r="AD3" s="2"/>
+      <c r="AE3" s="2"/>
+      <c r="AF3" s="2"/>
+      <c r="AG3" s="7"/>
+      <c r="AH3" s="7"/>
+      <c r="AI3" s="2"/>
+    </row>
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="2">
+        <v>35898</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="7"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="7"/>
+      <c r="T4" s="7"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="2"/>
+      <c r="W4" s="2"/>
+      <c r="X4" s="2"/>
+      <c r="Y4" s="2"/>
+      <c r="Z4" s="7"/>
+      <c r="AA4" s="7"/>
+      <c r="AB4" s="2"/>
+      <c r="AC4" s="2"/>
+      <c r="AD4" s="2"/>
+      <c r="AE4" s="2"/>
+      <c r="AF4" s="2"/>
+      <c r="AG4" s="7"/>
+      <c r="AH4" s="7"/>
+      <c r="AI4" s="2"/>
+    </row>
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="2">
+        <v>35898</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="7"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="7"/>
+      <c r="T5" s="7"/>
+      <c r="U5" s="2"/>
+      <c r="V5" s="2"/>
+      <c r="W5" s="2"/>
+      <c r="X5" s="2"/>
+      <c r="Y5" s="2"/>
+      <c r="Z5" s="7"/>
+      <c r="AA5" s="7"/>
+      <c r="AB5" s="2"/>
+      <c r="AC5" s="2"/>
+      <c r="AD5" s="2"/>
+      <c r="AE5" s="2"/>
+      <c r="AF5" s="2"/>
+      <c r="AG5" s="7"/>
+      <c r="AH5" s="7"/>
+      <c r="AI5" s="2"/>
+    </row>
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="2">
+        <v>52370</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="7"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
+      <c r="S6" s="7"/>
+      <c r="T6" s="7"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="2"/>
+      <c r="W6" s="2"/>
+      <c r="X6" s="2"/>
+      <c r="Y6" s="2"/>
+      <c r="Z6" s="7"/>
+      <c r="AA6" s="7"/>
+      <c r="AB6" s="2"/>
+      <c r="AC6" s="2"/>
+      <c r="AD6" s="2"/>
+      <c r="AE6" s="2"/>
+      <c r="AF6" s="2"/>
+      <c r="AG6" s="7"/>
+      <c r="AH6" s="7"/>
+      <c r="AI6" s="2"/>
+    </row>
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="2">
+        <v>33548</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="7"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="7"/>
+      <c r="T7" s="7"/>
+      <c r="U7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="V7" s="2"/>
+      <c r="W7" s="2"/>
+      <c r="X7" s="2"/>
+      <c r="Y7" s="2"/>
+      <c r="Z7" s="7"/>
+      <c r="AA7" s="7"/>
+      <c r="AB7" s="2"/>
+      <c r="AC7" s="2"/>
+      <c r="AD7" s="2"/>
+      <c r="AE7" s="2"/>
+      <c r="AF7" s="2"/>
+      <c r="AG7" s="7"/>
+      <c r="AH7" s="7"/>
+      <c r="AI7" s="2"/>
+    </row>
+    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2">
+        <v>44429</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="7"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="2"/>
+      <c r="R8" s="2"/>
+      <c r="S8" s="7"/>
+      <c r="T8" s="7"/>
+      <c r="U8" s="2"/>
+      <c r="V8" s="2"/>
+      <c r="W8" s="2"/>
+      <c r="X8" s="2"/>
+      <c r="Y8" s="2"/>
+      <c r="Z8" s="7"/>
+      <c r="AA8" s="7"/>
+      <c r="AB8" s="2"/>
+      <c r="AC8" s="2"/>
+      <c r="AD8" s="2"/>
+      <c r="AE8" s="2"/>
+      <c r="AF8" s="2"/>
+      <c r="AG8" s="7"/>
+      <c r="AH8" s="7"/>
+      <c r="AI8" s="2"/>
+    </row>
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A12" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <f>COUNTIF(F5:AI5,"WFO")</f>
+        <v>0</v>
       </c>
       <c r="C13" s="2">
         <f>COUNTIF(H5:AI5,"WFH")</f>
         <v>0</v>
       </c>
     </row>
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="2">
+        <f>COUNTIF(F7:AI7,"WFO")</f>
+        <v>0</v>
+      </c>
+      <c r="C14" s="2">
+        <f>COUNTIF(H7:AI7,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="2">
+        <f>COUNTIF(F8:AI8,"WFO")</f>
+        <v>0</v>
+      </c>
+      <c r="C15" s="2">
+        <f>COUNTIF(H8:AI8,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+  </mergeCells>
+  <phoneticPr fontId="8" type="noConversion"/>
+  <conditionalFormatting sqref="B13:B15">
+    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
+      <formula>11</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+      <formula>12</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+      <formula>12</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73C05419-3E5B-44D5-9A4D-7C953122A519}">
+  <dimension ref="A1:AJ15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="13" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="20" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="27" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="29" max="34" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1">
+        <v>46357</v>
+      </c>
+      <c r="G1" s="1">
+        <v>46358</v>
+      </c>
+      <c r="H1" s="1">
+        <v>46359</v>
+      </c>
+      <c r="I1" s="1">
+        <v>46360</v>
+      </c>
+      <c r="J1" s="1">
+        <v>46361</v>
+      </c>
+      <c r="K1" s="1">
+        <v>46362</v>
+      </c>
+      <c r="L1" s="1">
+        <v>46363</v>
+      </c>
+      <c r="M1" s="1">
+        <v>46364</v>
+      </c>
+      <c r="N1" s="1">
+        <v>46365</v>
+      </c>
+      <c r="O1" s="1">
+        <v>46366</v>
+      </c>
+      <c r="P1" s="1">
+        <v>46367</v>
+      </c>
+      <c r="Q1" s="1">
+        <v>46368</v>
+      </c>
+      <c r="R1" s="1">
+        <v>46369</v>
+      </c>
+      <c r="S1" s="1">
+        <v>46370</v>
+      </c>
+      <c r="T1" s="1">
+        <v>46371</v>
+      </c>
+      <c r="U1" s="1">
+        <v>46372</v>
+      </c>
+      <c r="V1" s="1">
+        <v>46373</v>
+      </c>
+      <c r="W1" s="1">
+        <v>46374</v>
+      </c>
+      <c r="X1" s="1">
+        <v>46375</v>
+      </c>
+      <c r="Y1" s="1">
+        <v>46376</v>
+      </c>
+      <c r="Z1" s="1">
+        <v>46377</v>
+      </c>
+      <c r="AA1" s="1">
+        <v>46378</v>
+      </c>
+      <c r="AB1" s="1">
+        <v>46379</v>
+      </c>
+      <c r="AC1" s="1">
+        <v>46380</v>
+      </c>
+      <c r="AD1" s="1">
+        <v>46381</v>
+      </c>
+      <c r="AE1" s="1">
+        <v>46382</v>
+      </c>
+      <c r="AF1" s="1">
+        <v>46383</v>
+      </c>
+      <c r="AG1" s="1">
+        <v>46384</v>
+      </c>
+      <c r="AH1" s="1">
+        <v>46385</v>
+      </c>
+      <c r="AI1" s="1">
+        <v>46386</v>
+      </c>
+      <c r="AJ1" s="1">
+        <v>46387</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="X2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="Z2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="AA2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AB2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="AC2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="AD2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="AE2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="AF2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="AG2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="AH2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AI2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="AJ2" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="2">
+        <v>51690</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="7"/>
+      <c r="R3" s="7"/>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
+      <c r="U3" s="2"/>
+      <c r="V3" s="2"/>
+      <c r="W3" s="2"/>
+      <c r="X3" s="7"/>
+      <c r="Y3" s="7"/>
+      <c r="Z3" s="2"/>
+      <c r="AA3" s="2"/>
+      <c r="AB3" s="2"/>
+      <c r="AC3" s="2"/>
+      <c r="AD3" s="2"/>
+      <c r="AE3" s="7"/>
+      <c r="AF3" s="7"/>
+      <c r="AG3" s="2"/>
+      <c r="AH3" s="2"/>
+      <c r="AI3" s="2"/>
+      <c r="AJ3" s="2"/>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="2">
+        <v>35898</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="7"/>
+      <c r="R4" s="7"/>
+      <c r="S4" s="2"/>
+      <c r="T4" s="2"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="2"/>
+      <c r="W4" s="2"/>
+      <c r="X4" s="7"/>
+      <c r="Y4" s="7"/>
+      <c r="Z4" s="2"/>
+      <c r="AA4" s="2"/>
+      <c r="AB4" s="2"/>
+      <c r="AC4" s="2"/>
+      <c r="AD4" s="2"/>
+      <c r="AE4" s="7"/>
+      <c r="AF4" s="7"/>
+      <c r="AG4" s="2"/>
+      <c r="AH4" s="2"/>
+      <c r="AI4" s="2"/>
+      <c r="AJ4" s="2"/>
+    </row>
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="2">
+        <v>35898</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="7"/>
+      <c r="R5" s="7"/>
+      <c r="S5" s="2"/>
+      <c r="T5" s="2"/>
+      <c r="U5" s="2"/>
+      <c r="V5" s="2"/>
+      <c r="W5" s="2"/>
+      <c r="X5" s="7"/>
+      <c r="Y5" s="7"/>
+      <c r="Z5" s="2"/>
+      <c r="AA5" s="2"/>
+      <c r="AB5" s="2"/>
+      <c r="AC5" s="2"/>
+      <c r="AD5" s="2"/>
+      <c r="AE5" s="7"/>
+      <c r="AF5" s="7"/>
+      <c r="AG5" s="2"/>
+      <c r="AH5" s="2"/>
+      <c r="AI5" s="2"/>
+      <c r="AJ5" s="2"/>
+    </row>
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="2">
+        <v>52370</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="7"/>
+      <c r="R6" s="7"/>
+      <c r="S6" s="2"/>
+      <c r="T6" s="2"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="2"/>
+      <c r="W6" s="2"/>
+      <c r="X6" s="7"/>
+      <c r="Y6" s="7"/>
+      <c r="Z6" s="2"/>
+      <c r="AA6" s="2"/>
+      <c r="AB6" s="2"/>
+      <c r="AC6" s="2"/>
+      <c r="AD6" s="2"/>
+      <c r="AE6" s="7"/>
+      <c r="AF6" s="7"/>
+      <c r="AG6" s="2"/>
+      <c r="AH6" s="2"/>
+      <c r="AI6" s="2"/>
+      <c r="AJ6" s="2"/>
+    </row>
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="2">
+        <v>33548</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="7"/>
+      <c r="R7" s="7"/>
+      <c r="S7" s="2"/>
+      <c r="T7" s="2"/>
+      <c r="U7" s="2"/>
+      <c r="V7" s="2"/>
+      <c r="W7" s="2"/>
+      <c r="X7" s="7"/>
+      <c r="Y7" s="7"/>
+      <c r="Z7" s="2"/>
+      <c r="AA7" s="2"/>
+      <c r="AB7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="AC7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="AD7" s="2"/>
+      <c r="AE7" s="7"/>
+      <c r="AF7" s="7"/>
+      <c r="AG7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="AH7" s="2"/>
+      <c r="AI7" s="2"/>
+      <c r="AJ7" s="2"/>
+    </row>
+    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2">
+        <v>44429</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="7"/>
+      <c r="R8" s="7"/>
+      <c r="S8" s="2"/>
+      <c r="T8" s="2"/>
+      <c r="U8" s="2"/>
+      <c r="V8" s="2"/>
+      <c r="W8" s="2"/>
+      <c r="X8" s="7"/>
+      <c r="Y8" s="7"/>
+      <c r="Z8" s="2"/>
+      <c r="AA8" s="2"/>
+      <c r="AB8" s="2"/>
+      <c r="AC8" s="2"/>
+      <c r="AD8" s="2"/>
+      <c r="AE8" s="7"/>
+      <c r="AF8" s="7"/>
+      <c r="AG8" s="2"/>
+      <c r="AH8" s="2"/>
+      <c r="AI8" s="2"/>
+      <c r="AJ8" s="2"/>
+    </row>
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A12" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <f>COUNTIF(F5:AI5,"WFO")</f>
+        <v>0</v>
+      </c>
+      <c r="C13" s="2">
+        <f>COUNTIF(H5:AI5,"WFH")</f>
+        <v>0</v>
+      </c>
+    </row>
     <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F7:AI7,"WFO")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(H7:AI7,"WFH")</f>
@@ -12599,11 +13889,11 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F8:AI8,"WFO")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(H8:AI8,"WFH")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -13330,10 +14620,10 @@
     <mergeCell ref="E1:E2"/>
   </mergeCells>
   <conditionalFormatting sqref="B10:B13">
-    <cfRule type="cellIs" dxfId="57" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="63" priority="1" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="62" priority="2" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14045,10 +15335,10 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B11:B14">
-    <cfRule type="cellIs" dxfId="55" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="61" priority="1" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="60" priority="2" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -14770,15 +16060,15 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B11:B14">
-    <cfRule type="cellIs" dxfId="53" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="59" priority="2" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="58" priority="4" operator="lessThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:B14">
-    <cfRule type="cellIs" dxfId="51" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="57" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15467,13 +16757,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="50" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="56" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="55" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="54" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16190,13 +17480,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="47" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="53" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="52" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="51" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16900,13 +18190,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="44" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="50" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="49" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="48" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17607,13 +18897,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B12:B15">
-    <cfRule type="cellIs" dxfId="41" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="47" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="46" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="45" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Daily attendance update - 2026-10-14
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C35E2714-EFAD-476D-8740-616CDCAAE9E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AC04204-79A0-43CC-9D7C-38242A05E396}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="19" activeTab="21" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="18" activeTab="21" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3386" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3424" uniqueCount="34">
   <si>
     <t>Person</t>
   </si>
@@ -158,6 +158,9 @@
   </si>
   <si>
     <t>Holiday</t>
+  </si>
+  <si>
+    <t>Ashish Chudaman Nagrikar</t>
   </si>
 </sst>
 </file>
@@ -11156,11 +11159,11 @@
         <v>30</v>
       </c>
       <c r="B13" s="4">
-        <f>COUNTIF(F3:AI3,"WFO")</f>
+        <f t="shared" ref="B13:B18" si="0">COUNTIF(F3:AI3,"WFO")</f>
         <v>13</v>
       </c>
       <c r="C13" s="2">
-        <f>COUNTIF(H3:AI3,"WFH")</f>
+        <f t="shared" ref="C13:C18" si="1">COUNTIF(H3:AI3,"WFH")</f>
         <v>8</v>
       </c>
     </row>
@@ -11169,11 +11172,11 @@
         <v>29</v>
       </c>
       <c r="B14" s="4">
-        <f>COUNTIF(F4:AI4,"WFO")</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C14" s="2">
-        <f>COUNTIF(H4:AI4,"WFH")</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
     </row>
@@ -11182,11 +11185,11 @@
         <v>12</v>
       </c>
       <c r="B15" s="2">
-        <f>COUNTIF(F5:AI5,"WFO")</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C15" s="2">
-        <f>COUNTIF(H5:AI5,"WFH")</f>
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
     </row>
@@ -11195,11 +11198,11 @@
         <v>31</v>
       </c>
       <c r="B16" s="2">
-        <f>COUNTIF(F6:AI6,"WFO")</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C16" s="2">
-        <f>COUNTIF(H6:AI6,"WFH")</f>
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
     </row>
@@ -11208,11 +11211,11 @@
         <v>19</v>
       </c>
       <c r="B17" s="2">
-        <f>COUNTIF(F7:AI7,"WFO")</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C17" s="2">
-        <f>COUNTIF(H7:AI7,"WFH")</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
     </row>
@@ -11221,11 +11224,11 @@
         <v>20</v>
       </c>
       <c r="B18" s="2">
-        <f>COUNTIF(F8:AI8,"WFO")</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C18" s="2">
-        <f>COUNTIF(H8:AI8,"WFH")</f>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
     </row>
@@ -11239,13 +11242,13 @@
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B15:B18">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="17" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="16" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11255,10 +11258,10 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A2B8991-FECB-4DED-BEB7-2ACC94684DF5}">
-  <dimension ref="A1:AJ18"/>
+  <dimension ref="A1:AJ19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
@@ -11532,7 +11535,9 @@
       <c r="R3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="S3" s="2"/>
+      <c r="S3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="T3" s="2"/>
       <c r="U3" s="2"/>
       <c r="V3" s="7"/>
@@ -11625,7 +11630,7 @@
     </row>
     <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="B5" s="2">
         <v>35898</v>
@@ -11639,9 +11644,7 @@
       <c r="E5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="5" t="s">
-        <v>17</v>
-      </c>
+      <c r="F5" s="5"/>
       <c r="G5" s="6" t="s">
         <v>28</v>
       </c>
@@ -11656,8 +11659,8 @@
       <c r="L5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="M5" s="6" t="s">
-        <v>24</v>
+      <c r="M5" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="N5" s="5" t="s">
         <v>17</v>
@@ -11670,7 +11673,9 @@
       <c r="R5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="S5" s="2"/>
+      <c r="S5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="T5" s="2"/>
       <c r="U5" s="2"/>
       <c r="V5" s="7"/>
@@ -11691,10 +11696,10 @@
     </row>
     <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="B6" s="2">
-        <v>52370</v>
+        <v>35898</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>13</v>
@@ -11722,8 +11727,8 @@
       <c r="L6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="M6" s="5" t="s">
-        <v>17</v>
+      <c r="M6" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="N6" s="5" t="s">
         <v>17</v>
@@ -11736,7 +11741,9 @@
       <c r="R6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="S6" s="2"/>
+      <c r="S6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="T6" s="2"/>
       <c r="U6" s="2"/>
       <c r="V6" s="7"/>
@@ -11757,10 +11764,10 @@
     </row>
     <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="B7" s="2">
-        <v>33548</v>
+        <v>52370</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>13</v>
@@ -11771,16 +11778,16 @@
       <c r="E7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>24</v>
+      <c r="F7" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="G7" s="6" t="s">
         <v>28</v>
       </c>
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
-      <c r="J7" s="6" t="s">
-        <v>24</v>
+      <c r="J7" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="K7" s="4" t="s">
         <v>16</v>
@@ -11788,8 +11795,8 @@
       <c r="L7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="M7" s="4" t="s">
-        <v>16</v>
+      <c r="M7" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="N7" s="5" t="s">
         <v>17</v>
@@ -11802,14 +11809,20 @@
       <c r="R7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="S7" s="2"/>
+      <c r="S7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="T7" s="2"/>
       <c r="U7" s="2"/>
       <c r="V7" s="7"/>
       <c r="W7" s="7"/>
       <c r="X7" s="2"/>
-      <c r="Y7" s="2"/>
-      <c r="Z7" s="2"/>
+      <c r="Y7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z7" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="AA7" s="2"/>
       <c r="AB7" s="2"/>
       <c r="AC7" s="7"/>
@@ -11823,10 +11836,10 @@
     </row>
     <row r="8" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8" s="2">
-        <v>44429</v>
+        <v>33548</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>13</v>
@@ -11835,18 +11848,18 @@
         <v>14</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="G8" s="6" t="s">
         <v>28</v>
       </c>
       <c r="H8" s="7"/>
       <c r="I8" s="7"/>
-      <c r="J8" s="5" t="s">
-        <v>17</v>
+      <c r="J8" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="K8" s="4" t="s">
         <v>16</v>
@@ -11868,14 +11881,14 @@
       <c r="R8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="S8" s="2"/>
+      <c r="S8" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="T8" s="2"/>
       <c r="U8" s="2"/>
       <c r="V8" s="7"/>
       <c r="W8" s="7"/>
-      <c r="X8" s="6" t="s">
-        <v>24</v>
-      </c>
+      <c r="X8" s="2"/>
       <c r="Y8" s="2"/>
       <c r="Z8" s="2"/>
       <c r="AA8" s="2"/>
@@ -11889,92 +11902,162 @@
       <c r="AI8" s="2"/>
       <c r="AJ8" s="7"/>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="2">
+        <v>44429</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="M9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="O9" s="7"/>
+      <c r="P9" s="7"/>
+      <c r="Q9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="R9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="S9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="T9" s="2"/>
+      <c r="U9" s="2"/>
+      <c r="V9" s="7"/>
+      <c r="W9" s="7"/>
+      <c r="X9" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="Y9" s="2"/>
+      <c r="Z9" s="2"/>
+      <c r="AA9" s="2"/>
+      <c r="AB9" s="2"/>
+      <c r="AC9" s="7"/>
+      <c r="AD9" s="7"/>
+      <c r="AE9" s="2"/>
+      <c r="AF9" s="2"/>
+      <c r="AG9" s="2"/>
+      <c r="AH9" s="2"/>
+      <c r="AI9" s="2"/>
+      <c r="AJ9" s="7"/>
+    </row>
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A13" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B14" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
         <v>6</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C14" s="2">
         <f>COUNTIF(H3:AI3,"WFH")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B15" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
         <v>4</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C15" s="2">
         <f>COUNTIF(H4:AI4,"WFH")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B15" s="2">
-        <f>COUNTIF(F5:AI5,"WFO")</f>
-        <v>5</v>
-      </c>
-      <c r="C15" s="2">
-        <f>COUNTIF(H5:AI5,"WFH")</f>
-        <v>1</v>
-      </c>
-    </row>
     <row r="16" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="B16" s="2">
-        <f>COUNTIF(F6:AI6,"WFO")</f>
+        <f t="shared" ref="B16:B19" si="0">COUNTIF(F6:AI6,"WFO")</f>
         <v>5</v>
       </c>
       <c r="C16" s="2">
-        <f>COUNTIF(H6:AI6,"WFH")</f>
+        <f t="shared" ref="C16:C19" si="1">COUNTIF(H6:AI6,"WFH")</f>
         <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="B17" s="2">
-        <f>COUNTIF(F7:AI7,"WFO")</f>
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>6</v>
       </c>
       <c r="C17" s="2">
-        <f>COUNTIF(H7:AI7,"WFH")</f>
-        <v>1</v>
+        <f t="shared" si="1"/>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="2">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="C18" s="2">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="2">
-        <f>COUNTIF(F8:AI8,"WFO")</f>
-        <v>5</v>
-      </c>
-      <c r="C18" s="2">
-        <f>COUNTIF(H8:AI8,"WFH")</f>
+      <c r="B19" s="2">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="C19" s="2">
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
     </row>
@@ -11987,25 +12070,14 @@
     <mergeCell ref="E1:E2"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
-  <conditionalFormatting sqref="B15:B18">
-    <cfRule type="cellIs" dxfId="14" priority="4" operator="greaterThan">
+  <conditionalFormatting sqref="B14:B19">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="5" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="6" operator="greaterThan">
-      <formula>12</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B13:B14">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
-      <formula>11</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
-      <formula>12</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12015,7 +12087,7 @@
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4E8A644-1993-49C0-933B-42395C786DC4}">
-  <dimension ref="A1:AI15"/>
+  <dimension ref="A1:AI18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
@@ -12264,7 +12336,9 @@
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
       <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
+      <c r="O3" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
       <c r="R3" s="2"/>
@@ -12311,7 +12385,9 @@
       <c r="L4" s="7"/>
       <c r="M4" s="7"/>
       <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
+      <c r="O4" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
       <c r="R4" s="2"/>
@@ -12362,7 +12438,9 @@
       <c r="N5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="O5" s="2"/>
+      <c r="O5" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
       <c r="R5" s="2"/>
@@ -12409,7 +12487,9 @@
       <c r="L6" s="7"/>
       <c r="M6" s="7"/>
       <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
+      <c r="O6" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
       <c r="R6" s="2"/>
@@ -12456,7 +12536,9 @@
       <c r="L7" s="7"/>
       <c r="M7" s="7"/>
       <c r="N7" s="2"/>
-      <c r="O7" s="2"/>
+      <c r="O7" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="P7" s="2"/>
       <c r="Q7" s="2"/>
       <c r="R7" s="2"/>
@@ -12507,7 +12589,9 @@
       <c r="N8" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="O8" s="2"/>
+      <c r="O8" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="P8" s="2"/>
       <c r="Q8" s="2"/>
       <c r="R8" s="2"/>
@@ -12542,40 +12626,79 @@
     </row>
     <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="B13" s="2">
-        <f>COUNTIF(F5:AI5,"WFO")</f>
+        <f t="shared" ref="B13:B18" si="0">COUNTIF(F3:AI3,"WFO")</f>
         <v>0</v>
       </c>
       <c r="C13" s="2">
-        <f>COUNTIF(H5:AI5,"WFH")</f>
+        <f t="shared" ref="C13:C18" si="1">COUNTIF(H3:AI3,"WFH")</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="B14" s="2">
-        <f>COUNTIF(F7:AI7,"WFO")</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="C14" s="2">
-        <f>COUNTIF(H7:AI7,"WFH")</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="C15" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="C16" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="C17" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="2">
-        <f>COUNTIF(F8:AI8,"WFO")</f>
+      <c r="B18" s="2">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="C15" s="2">
-        <f>COUNTIF(H8:AI8,"WFH")</f>
+      <c r="C18" s="2">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -12588,14 +12711,14 @@
     <mergeCell ref="E1:E2"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
-  <conditionalFormatting sqref="B13:B15">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="greaterThan">
+  <conditionalFormatting sqref="B13:B18">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12605,7 +12728,7 @@
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73C05419-3E5B-44D5-9A4D-7C953122A519}">
-  <dimension ref="A1:AJ15"/>
+  <dimension ref="A1:AJ18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
@@ -12876,7 +12999,9 @@
       <c r="AA3" s="2"/>
       <c r="AB3" s="2"/>
       <c r="AC3" s="2"/>
-      <c r="AD3" s="2"/>
+      <c r="AD3" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="AE3" s="7"/>
       <c r="AF3" s="7"/>
       <c r="AG3" s="2"/>
@@ -12924,7 +13049,9 @@
       <c r="AA4" s="2"/>
       <c r="AB4" s="2"/>
       <c r="AC4" s="2"/>
-      <c r="AD4" s="2"/>
+      <c r="AD4" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="AE4" s="7"/>
       <c r="AF4" s="7"/>
       <c r="AG4" s="2"/>
@@ -12980,7 +13107,9 @@
       <c r="AA5" s="2"/>
       <c r="AB5" s="2"/>
       <c r="AC5" s="2"/>
-      <c r="AD5" s="2"/>
+      <c r="AD5" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="AE5" s="7"/>
       <c r="AF5" s="7"/>
       <c r="AG5" s="2"/>
@@ -13028,7 +13157,9 @@
       <c r="AA6" s="2"/>
       <c r="AB6" s="2"/>
       <c r="AC6" s="2"/>
-      <c r="AD6" s="2"/>
+      <c r="AD6" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="AE6" s="7"/>
       <c r="AF6" s="7"/>
       <c r="AG6" s="2"/>
@@ -13080,7 +13211,9 @@
       <c r="AC7" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="AD7" s="2"/>
+      <c r="AD7" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="AE7" s="7"/>
       <c r="AF7" s="7"/>
       <c r="AG7" s="6" t="s">
@@ -13138,7 +13271,9 @@
       <c r="AC8" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="AD8" s="2"/>
+      <c r="AD8" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="AE8" s="7"/>
       <c r="AF8" s="7"/>
       <c r="AG8" s="6" t="s">
@@ -13167,40 +13302,79 @@
     </row>
     <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="B13" s="2">
-        <f>COUNTIF(F5:AI5,"WFO")</f>
+        <f t="shared" ref="B13:B18" si="0">COUNTIF(F3:AI3,"WFO")</f>
         <v>0</v>
       </c>
       <c r="C13" s="2">
-        <f>COUNTIF(H5:AI5,"WFH")</f>
+        <f t="shared" ref="C13:C18" si="1">COUNTIF(H3:AI3,"WFH")</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="B14" s="2">
-        <f>COUNTIF(F7:AI7,"WFO")</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="C14" s="2">
-        <f>COUNTIF(H7:AI7,"WFH")</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="C15" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="C16" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="2">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="C17" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="2">
-        <f>COUNTIF(F8:AI8,"WFO")</f>
+      <c r="B18" s="2">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="C15" s="2">
-        <f>COUNTIF(H8:AI8,"WFH")</f>
+      <c r="C18" s="2">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -13213,14 +13387,14 @@
     <mergeCell ref="E1:E2"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
-  <conditionalFormatting sqref="B13:B15">
-    <cfRule type="cellIs" dxfId="8" priority="1" operator="greaterThan">
+  <conditionalFormatting sqref="B13:B18">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
       <formula>11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="2" operator="lessThan">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
       <formula>12</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThan">
       <formula>12</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Daily attendance update - 2026-10-15
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5491CD8-2B25-4C4C-B854-6C6A6A5F9160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60F8219C-F07B-41D5-B6F0-D284D9A03DE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="19" activeTab="21" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="19" activeTab="21" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3446" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3452" uniqueCount="34">
   <si>
     <t>Person</t>
   </si>
@@ -11478,7 +11478,9 @@
       <c r="S3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="T3" s="2"/>
+      <c r="T3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="U3" s="2"/>
       <c r="V3" s="7"/>
       <c r="W3" s="7"/>
@@ -11618,7 +11620,9 @@
       <c r="S5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="T5" s="2"/>
+      <c r="T5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="U5" s="2"/>
       <c r="V5" s="7"/>
       <c r="W5" s="7"/>
@@ -11694,7 +11698,9 @@
       <c r="S6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="T6" s="2"/>
+      <c r="T6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="U6" s="2"/>
       <c r="V6" s="7"/>
       <c r="W6" s="7"/>
@@ -11762,7 +11768,9 @@
       <c r="S7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="T7" s="2"/>
+      <c r="T7" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="U7" s="2"/>
       <c r="V7" s="7"/>
       <c r="W7" s="7"/>
@@ -11834,7 +11842,9 @@
       <c r="S8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="T8" s="2"/>
+      <c r="T8" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="U8" s="2"/>
       <c r="V8" s="7"/>
       <c r="W8" s="7"/>
@@ -11902,7 +11912,9 @@
       <c r="S9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="T9" s="2"/>
+      <c r="T9" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="U9" s="2"/>
       <c r="V9" s="7"/>
       <c r="W9" s="7"/>
@@ -11943,7 +11955,7 @@
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(H3:AI3,"WFH")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:36" x14ac:dyDescent="0.25">
@@ -11969,7 +11981,7 @@
       </c>
       <c r="C16" s="2">
         <f t="shared" ref="C16:C19" si="1">COUNTIF(H6:AI6,"WFH")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -11982,7 +11994,7 @@
       </c>
       <c r="C17" s="2">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -11991,7 +12003,7 @@
       </c>
       <c r="B18" s="2">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C18" s="2">
         <f t="shared" si="1"/>
@@ -12008,7 +12020,7 @@
       </c>
       <c r="C19" s="2">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-10-18
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BFE71B4-07BB-4D8F-BB90-6A4D165C45D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04E3C494-CCC5-4293-8597-7E486044E872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="19" activeTab="23" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="21" activeTab="21" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3457" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3469" uniqueCount="34">
   <si>
     <t>Person</t>
   </si>
@@ -1357,31 +1357,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27991520-C614-4BFB-ADD8-628FF075C04B}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="9.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -1491,7 +1491,7 @@
         <v>45688</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -1591,7 +1591,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1685,7 +1685,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -1779,7 +1779,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -1873,7 +1873,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -1967,7 +1967,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -2061,7 +2061,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -2072,7 +2072,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -2085,7 +2085,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -2098,7 +2098,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -2111,7 +2111,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -2124,7 +2124,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -2153,30 +2153,30 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{826FC1B3-53E6-4D35-9223-A0DEC05CDA48}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="19" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="24" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="28" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="12" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="19" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="21" max="24" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="28" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2286,7 +2286,7 @@
         <v>45961</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2386,7 +2386,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2480,7 +2480,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -2574,7 +2574,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2668,7 +2668,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -2762,7 +2762,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2800,7 +2800,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -2811,7 +2811,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -2824,7 +2824,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -2837,7 +2837,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -2850,7 +2850,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -2890,26 +2890,26 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C42BC0F2-E7C0-48B4-8AB8-C4D08FDA0656}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -3016,7 +3016,7 @@
         <v>45991</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3113,7 +3113,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -3200,7 +3200,7 @@
       <c r="AH3" s="7"/>
       <c r="AI3" s="7"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -3287,7 +3287,7 @@
       <c r="AH4" s="7"/>
       <c r="AI4" s="7"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3374,7 +3374,7 @@
       <c r="AH5" s="7"/>
       <c r="AI5" s="7"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3461,7 +3461,7 @@
       <c r="AH6" s="7"/>
       <c r="AI6" s="7"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -3498,7 +3498,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -3509,7 +3509,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -3522,7 +3522,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -3535,7 +3535,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -3548,7 +3548,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -3588,27 +3588,27 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{988C623D-E1BD-4FE8-8DE5-A86BDEB0A522}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -3718,7 +3718,7 @@
         <v>46022</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3818,7 +3818,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -3912,7 +3912,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -4006,7 +4006,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4100,7 +4100,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -4194,7 +4194,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4232,7 +4232,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -4243,7 +4243,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -4256,7 +4256,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -4269,7 +4269,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4282,7 +4282,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4322,27 +4322,27 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9E71A27-DC0F-4421-B295-A887695B49EA}">
   <dimension ref="A1:AJ13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -4452,7 +4452,7 @@
         <v>46053</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -4552,7 +4552,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -4644,7 +4644,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -4736,7 +4736,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4828,7 +4828,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -4866,7 +4866,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="2"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
         <v>1</v>
       </c>
@@ -4877,7 +4877,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -4890,7 +4890,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -4903,7 +4903,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -4943,26 +4943,26 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F94C369-A483-4243-8B30-4AC8F8C2C920}">
   <dimension ref="A1:AG12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -5063,7 +5063,7 @@
         <v>46081</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -5154,7 +5154,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5239,7 +5239,7 @@
       </c>
       <c r="AG3" s="7"/>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5324,7 +5324,7 @@
       </c>
       <c r="AG4" s="7"/>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5409,7 +5409,7 @@
       </c>
       <c r="AG5" s="7"/>
     </row>
-    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>1</v>
       </c>
@@ -5420,7 +5420,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -5433,7 +5433,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -5446,7 +5446,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -5486,27 +5486,27 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72154BF-0805-461D-B9A5-E64EDBF4FEB9}">
   <dimension ref="A1:AJ12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -5616,7 +5616,7 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -5716,7 +5716,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5808,7 +5808,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5900,7 +5900,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5992,7 +5992,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>1</v>
       </c>
@@ -6003,7 +6003,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -6016,7 +6016,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -6029,7 +6029,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -6069,27 +6069,27 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF130E33-32AF-452B-AEB5-3A35260DB102}">
   <dimension ref="A1:AI12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="35" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="35" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6196,7 +6196,7 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -6293,7 +6293,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -6384,7 +6384,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -6475,7 +6475,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -6566,7 +6566,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>1</v>
       </c>
@@ -6577,7 +6577,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -6590,7 +6590,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -6603,7 +6603,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -6643,29 +6643,29 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97DA7DA3-001B-413F-BA22-DC9827945C1D}">
   <dimension ref="A1:AJ12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="19" max="24" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="26" max="31" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="33" max="36" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="17" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="19" max="24" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="26" max="31" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="33" max="36" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6775,7 +6775,7 @@
         <v>46173</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -6875,7 +6875,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -6965,7 +6965,7 @@
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -7055,7 +7055,7 @@
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -7145,7 +7145,7 @@
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>1</v>
       </c>
@@ -7156,7 +7156,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -7169,7 +7169,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -7182,7 +7182,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -7222,27 +7222,27 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{934EE78C-1B04-4E2F-8C73-18B0A1ECFFAE}">
   <dimension ref="A1:AI13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="21" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="23" max="28" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="30" max="35" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="21" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="23" max="28" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="30" max="35" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -7349,7 +7349,7 @@
         <v>46203</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -7446,7 +7446,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>29</v>
       </c>
@@ -7537,7 +7537,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -7628,7 +7628,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
@@ -7719,7 +7719,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -7810,7 +7810,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
         <v>1</v>
       </c>
@@ -7821,7 +7821,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -7834,7 +7834,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -7847,7 +7847,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -7887,27 +7887,27 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77C449D2-15A1-404E-9EF3-800FA95F32E2}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="21" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="23" max="28" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="30" max="35" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="21" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="23" max="28" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="30" max="35" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -8017,7 +8017,7 @@
         <v>46234</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -8117,7 +8117,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -8205,7 +8205,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -8299,7 +8299,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -8393,7 +8393,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
@@ -8461,7 +8461,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -8555,7 +8555,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -8649,7 +8649,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
         <v>1</v>
       </c>
@@ -8660,7 +8660,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
@@ -8673,7 +8673,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>19</v>
       </c>
@@ -8686,7 +8686,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -8727,30 +8727,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A6D4258-8D1D-40C7-BB83-4C4F9F65CC0B}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -8851,7 +8851,7 @@
         <v>45716</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -8942,7 +8942,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -9027,7 +9027,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -9114,7 +9114,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -9201,7 +9201,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -9286,7 +9286,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -9371,7 +9371,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -9382,7 +9382,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -9395,7 +9395,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -9408,7 +9408,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -9421,7 +9421,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -9434,7 +9434,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -9462,29 +9462,29 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F59B1450-F750-4AAF-92F1-86BC63885A84}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="12.85546875" customWidth="1"/>
-    <col min="8" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="36" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="12.81640625" customWidth="1"/>
+    <col min="8" max="9" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="36" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9594,7 +9594,7 @@
         <v>46265</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -9694,7 +9694,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -9784,7 +9784,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -9874,7 +9874,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -9964,7 +9964,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
@@ -10054,7 +10054,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -10144,7 +10144,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -10234,7 +10234,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
         <v>1</v>
       </c>
@@ -10245,7 +10245,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
@@ -10258,7 +10258,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>19</v>
       </c>
@@ -10271,7 +10271,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -10311,29 +10311,29 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57075C38-32AC-4EA3-9612-A4A3D80F7093}">
   <dimension ref="A1:AI18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="12.85546875" customWidth="1"/>
-    <col min="8" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="12.81640625" customWidth="1"/>
+    <col min="8" max="9" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -10440,7 +10440,7 @@
         <v>46295</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -10537,7 +10537,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -10628,7 +10628,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -10719,7 +10719,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -10810,7 +10810,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
@@ -10901,7 +10901,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -10992,7 +10992,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -11083,7 +11083,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
         <v>1</v>
       </c>
@@ -11094,7 +11094,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>30</v>
       </c>
@@ -11107,7 +11107,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>29</v>
       </c>
@@ -11120,7 +11120,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>12</v>
       </c>
@@ -11133,7 +11133,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>31</v>
       </c>
@@ -11146,7 +11146,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>19</v>
       </c>
@@ -11159,7 +11159,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -11199,26 +11199,26 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A2B8991-FECB-4DED-BEB7-2ACC94684DF5}">
   <dimension ref="A1:AJ19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="11" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="18" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="25" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="27" max="32" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="11" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="18" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="20" max="25" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="27" max="32" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -11328,7 +11328,7 @@
         <v>46326</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -11428,7 +11428,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -11481,10 +11481,14 @@
       <c r="T3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="U3" s="2"/>
+      <c r="U3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="V3" s="7"/>
       <c r="W3" s="7"/>
-      <c r="X3" s="2"/>
+      <c r="X3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="Y3" s="2"/>
       <c r="Z3" s="2"/>
       <c r="AA3" s="2"/>
@@ -11498,7 +11502,7 @@
       <c r="AI3" s="2"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -11580,7 +11584,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>33</v>
       </c>
@@ -11633,10 +11637,14 @@
       <c r="T5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="U5" s="2"/>
+      <c r="U5" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="V5" s="7"/>
       <c r="W5" s="7"/>
-      <c r="X5" s="2"/>
+      <c r="X5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="Y5" s="2"/>
       <c r="Z5" s="6" t="s">
         <v>24</v>
@@ -11658,7 +11666,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
@@ -11711,10 +11719,14 @@
       <c r="T6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="U6" s="2"/>
+      <c r="U6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="V6" s="7"/>
       <c r="W6" s="7"/>
-      <c r="X6" s="2"/>
+      <c r="X6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="Y6" s="2"/>
       <c r="Z6" s="2"/>
       <c r="AA6" s="2"/>
@@ -11728,7 +11740,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>31</v>
       </c>
@@ -11781,10 +11793,14 @@
       <c r="T7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="U7" s="2"/>
+      <c r="U7" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="V7" s="7"/>
       <c r="W7" s="7"/>
-      <c r="X7" s="2"/>
+      <c r="X7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="Y7" s="6" t="s">
         <v>24</v>
       </c>
@@ -11802,7 +11818,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="7"/>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
@@ -11855,10 +11871,14 @@
       <c r="T8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="U8" s="2"/>
+      <c r="U8" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="V8" s="7"/>
       <c r="W8" s="7"/>
-      <c r="X8" s="2"/>
+      <c r="X8" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="Y8" s="2"/>
       <c r="Z8" s="2"/>
       <c r="AA8" s="2"/>
@@ -11872,7 +11892,7 @@
       <c r="AI8" s="2"/>
       <c r="AJ8" s="7"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -11925,13 +11945,17 @@
       <c r="T9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="U9" s="2"/>
+      <c r="U9" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="V9" s="7"/>
       <c r="W9" s="7"/>
-      <c r="X9" s="6" t="s">
+      <c r="X9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Y9" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="Y9" s="2"/>
       <c r="Z9" s="2"/>
       <c r="AA9" s="2"/>
       <c r="AB9" s="2"/>
@@ -11944,7 +11968,7 @@
       <c r="AI9" s="2"/>
       <c r="AJ9" s="7"/>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
         <v>1</v>
       </c>
@@ -11955,20 +11979,20 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(H3:AI3,"WFH")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>29</v>
       </c>
@@ -11981,56 +12005,56 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B16" s="2">
         <f t="shared" ref="B16:B19" si="0">COUNTIF(F6:AI6,"WFO")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C16" s="2">
         <f t="shared" ref="C16:C19" si="1">COUNTIF(H6:AI6,"WFH")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B17" s="2">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C17" s="2">
         <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B18" s="2">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C18" s="2">
         <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B19" s="2">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C19" s="2">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -12060,26 +12084,26 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4E8A644-1993-49C0-933B-42395C786DC4}">
   <dimension ref="A1:AI19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="22" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="24" max="29" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="31" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="17" max="22" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="24" max="29" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="31" max="35" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -12186,7 +12210,7 @@
         <v>46356</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -12283,7 +12307,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -12332,7 +12356,7 @@
       <c r="AH3" s="7"/>
       <c r="AI3" s="2"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -12381,7 +12405,7 @@
       <c r="AH4" s="7"/>
       <c r="AI4" s="2"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>33</v>
       </c>
@@ -12438,7 +12462,7 @@
       <c r="AH5" s="7"/>
       <c r="AI5" s="2"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
@@ -12491,7 +12515,7 @@
       <c r="AH6" s="7"/>
       <c r="AI6" s="2"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>31</v>
       </c>
@@ -12540,7 +12564,7 @@
       <c r="AH7" s="7"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
@@ -12591,7 +12615,7 @@
       <c r="AH8" s="7"/>
       <c r="AI8" s="2"/>
     </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -12642,7 +12666,7 @@
       <c r="AH9" s="7"/>
       <c r="AI9" s="2"/>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
         <v>1</v>
       </c>
@@ -12653,7 +12677,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>30</v>
       </c>
@@ -12666,7 +12690,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>29</v>
       </c>
@@ -12679,7 +12703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
@@ -12692,7 +12716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>31</v>
       </c>
@@ -12705,7 +12729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>19</v>
       </c>
@@ -12718,7 +12742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -12758,27 +12782,27 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73C05419-3E5B-44D5-9A4D-7C953122A519}">
   <dimension ref="A1:AJ19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="13" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="20" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="22" max="27" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="29" max="34" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="13" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="15" max="20" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="22" max="27" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="29" max="34" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -12888,7 +12912,7 @@
         <v>46387</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -12988,7 +13012,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -13038,7 +13062,7 @@
       <c r="AI3" s="2"/>
       <c r="AJ3" s="2"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -13088,7 +13112,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="2"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>33</v>
       </c>
@@ -13144,7 +13168,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="2"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
@@ -13202,7 +13226,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="2"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>31</v>
       </c>
@@ -13252,7 +13276,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
@@ -13308,7 +13332,7 @@
       <c r="AI8" s="2"/>
       <c r="AJ8" s="2"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -13374,7 +13398,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
         <v>1</v>
       </c>
@@ -13385,7 +13409,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>30</v>
       </c>
@@ -13398,7 +13422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>29</v>
       </c>
@@ -13411,7 +13435,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
@@ -13424,7 +13448,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>31</v>
       </c>
@@ -13437,7 +13461,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>19</v>
       </c>
@@ -13450,7 +13474,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -13491,28 +13515,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E625ADA5-2D1E-431C-8817-0E3A7680EE75}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AJ13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="10.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -13622,7 +13646,7 @@
         <v>45747</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -13722,7 +13746,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -13812,7 +13836,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -13900,7 +13924,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="13"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -13988,7 +14012,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="13"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -14076,7 +14100,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="13"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -14114,7 +14138,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="14"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
         <v>1</v>
       </c>
@@ -14125,7 +14149,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -14138,7 +14162,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -14151,7 +14175,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -14164,7 +14188,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
@@ -14202,29 +14226,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61D25C68-D147-4871-A2A8-2CD748E8464B}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:AI14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -14331,7 +14355,7 @@
         <v>45777</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -14428,7 +14452,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -14519,7 +14543,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -14610,7 +14634,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -14701,7 +14725,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -14792,7 +14816,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -14829,7 +14853,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -14840,7 +14864,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -14853,7 +14877,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -14866,7 +14890,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -14879,7 +14903,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -14917,29 +14941,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460154BA-7A2B-4633-BD09-4305E2926D5D}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:AJ14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="18" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="25" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="27" max="32" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="15" max="18" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="20" max="25" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="27" max="32" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -15049,7 +15073,7 @@
         <v>45808</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -15149,7 +15173,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -15241,7 +15265,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -15333,7 +15357,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -15425,7 +15449,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -15517,7 +15541,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -15554,7 +15578,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -15565,7 +15589,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -15578,7 +15602,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -15591,7 +15615,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -15604,7 +15628,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -15646,15 +15670,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55B0C082-0457-4696-978D-1BE2DD3075D3}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -15761,7 +15785,7 @@
         <v>45838</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -15858,7 +15882,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -15947,7 +15971,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -16036,7 +16060,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -16125,7 +16149,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -16214,7 +16238,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -16251,7 +16275,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
         <v>1</v>
       </c>
@@ -16262,7 +16286,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -16275,7 +16299,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -16288,7 +16312,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -16301,7 +16325,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -16341,17 +16365,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6D2793F-73F1-4265-B1CF-8D693D22CC02}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -16461,7 +16485,7 @@
         <v>45869</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -16561,7 +16585,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -16655,7 +16679,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -16749,7 +16773,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -16843,7 +16867,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -16937,7 +16961,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -16974,7 +16998,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -16985,7 +17009,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -16998,7 +17022,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -17011,7 +17035,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -17024,7 +17048,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -17064,18 +17088,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F16C68-A443-46CF-B7FA-2968469C0FB5}">
   <dimension ref="A1:AK15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -17186,7 +17210,7 @@
       </c>
       <c r="AK1" s="1"/>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -17286,7 +17310,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -17376,7 +17400,7 @@
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -17466,7 +17490,7 @@
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -17556,7 +17580,7 @@
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -17646,7 +17670,7 @@
       <c r="AI6" s="7"/>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -17684,7 +17708,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -17695,7 +17719,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -17708,7 +17732,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -17721,7 +17745,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -17734,7 +17758,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -17774,19 +17798,19 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED7CEAED-F464-426C-A766-484A87191C7F}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -17893,7 +17917,7 @@
         <v>45930</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -17990,7 +18014,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -18081,7 +18105,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -18172,7 +18196,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -18263,7 +18287,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -18354,7 +18378,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -18391,7 +18415,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -18402,7 +18426,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -18415,7 +18439,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -18428,7 +18452,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -18441,7 +18465,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
Daily attendance update - 2026-10-19
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04E3C494-CCC5-4293-8597-7E486044E872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B4975DF-5F4A-4B2D-BDA8-07D5F68A1016}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="21" activeTab="21" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="21" activeTab="21" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3469" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3470" uniqueCount="34">
   <si>
     <t>Person</t>
   </si>
@@ -1357,31 +1357,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27991520-C614-4BFB-ADD8-628FF075C04B}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -1491,7 +1491,7 @@
         <v>45688</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -1591,7 +1591,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1685,7 +1685,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -1779,7 +1779,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -1873,7 +1873,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -1967,7 +1967,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -2061,7 +2061,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -2072,7 +2072,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -2085,7 +2085,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -2098,7 +2098,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -2111,7 +2111,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -2124,7 +2124,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -2153,30 +2153,30 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{826FC1B3-53E6-4D35-9223-A0DEC05CDA48}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="12" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="19" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="21" max="24" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="28" max="33" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="19" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="24" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="28" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2286,7 +2286,7 @@
         <v>45961</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2386,7 +2386,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2480,7 +2480,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -2574,7 +2574,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2668,7 +2668,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -2762,7 +2762,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2800,7 +2800,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -2811,7 +2811,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -2824,7 +2824,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -2837,7 +2837,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -2850,7 +2850,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -2890,26 +2890,26 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C42BC0F2-E7C0-48B4-8AB8-C4D08FDA0656}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -3016,7 +3016,7 @@
         <v>45991</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3113,7 +3113,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -3200,7 +3200,7 @@
       <c r="AH3" s="7"/>
       <c r="AI3" s="7"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -3287,7 +3287,7 @@
       <c r="AH4" s="7"/>
       <c r="AI4" s="7"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3374,7 +3374,7 @@
       <c r="AH5" s="7"/>
       <c r="AI5" s="7"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3461,7 +3461,7 @@
       <c r="AH6" s="7"/>
       <c r="AI6" s="7"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -3498,7 +3498,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -3509,7 +3509,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -3522,7 +3522,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -3535,7 +3535,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -3548,7 +3548,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -3588,27 +3588,27 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{988C623D-E1BD-4FE8-8DE5-A86BDEB0A522}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -3718,7 +3718,7 @@
         <v>46022</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3818,7 +3818,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -3912,7 +3912,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -4006,7 +4006,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4100,7 +4100,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -4194,7 +4194,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4232,7 +4232,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -4243,7 +4243,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -4256,7 +4256,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -4269,7 +4269,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4282,7 +4282,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4322,27 +4322,27 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9E71A27-DC0F-4421-B295-A887695B49EA}">
   <dimension ref="A1:AJ13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -4452,7 +4452,7 @@
         <v>46053</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -4552,7 +4552,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -4644,7 +4644,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -4736,7 +4736,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4828,7 +4828,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -4866,7 +4866,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="2"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>1</v>
       </c>
@@ -4877,7 +4877,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -4890,7 +4890,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -4903,7 +4903,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -4943,26 +4943,26 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F94C369-A483-4243-8B30-4AC8F8C2C920}">
   <dimension ref="A1:AG12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -5063,7 +5063,7 @@
         <v>46081</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -5154,7 +5154,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5239,7 +5239,7 @@
       </c>
       <c r="AG3" s="7"/>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5324,7 +5324,7 @@
       </c>
       <c r="AG4" s="7"/>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5409,7 +5409,7 @@
       </c>
       <c r="AG5" s="7"/>
     </row>
-    <row r="9" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>1</v>
       </c>
@@ -5420,7 +5420,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -5433,7 +5433,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -5446,7 +5446,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -5486,27 +5486,27 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72154BF-0805-461D-B9A5-E64EDBF4FEB9}">
   <dimension ref="A1:AJ12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -5616,7 +5616,7 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -5716,7 +5716,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5808,7 +5808,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5900,7 +5900,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5992,7 +5992,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>1</v>
       </c>
@@ -6003,7 +6003,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -6016,7 +6016,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -6029,7 +6029,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -6069,27 +6069,27 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF130E33-32AF-452B-AEB5-3A35260DB102}">
   <dimension ref="A1:AI12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="34" max="35" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="35" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6196,7 +6196,7 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -6293,7 +6293,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -6384,7 +6384,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -6475,7 +6475,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -6566,7 +6566,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>1</v>
       </c>
@@ -6577,7 +6577,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -6590,7 +6590,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -6603,7 +6603,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -6643,29 +6643,29 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97DA7DA3-001B-413F-BA22-DC9827945C1D}">
   <dimension ref="A1:AJ12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="19" max="24" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="26" max="31" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="33" max="36" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="17" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="24" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="26" max="31" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="33" max="36" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6775,7 +6775,7 @@
         <v>46173</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -6875,7 +6875,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -6965,7 +6965,7 @@
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -7055,7 +7055,7 @@
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -7145,7 +7145,7 @@
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>1</v>
       </c>
@@ -7156,7 +7156,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -7169,7 +7169,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -7182,7 +7182,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -7222,27 +7222,27 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{934EE78C-1B04-4E2F-8C73-18B0A1ECFFAE}">
   <dimension ref="A1:AI13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="16" max="21" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="23" max="28" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="30" max="35" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="21" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="28" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="30" max="35" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -7349,7 +7349,7 @@
         <v>46203</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -7446,7 +7446,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>29</v>
       </c>
@@ -7537,7 +7537,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -7628,7 +7628,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
@@ -7719,7 +7719,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -7810,7 +7810,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>1</v>
       </c>
@@ -7821,7 +7821,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -7834,7 +7834,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -7847,7 +7847,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -7887,27 +7887,27 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77C449D2-15A1-404E-9EF3-800FA95F32E2}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="16" max="21" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="23" max="28" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="30" max="35" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="21" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="23" max="28" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="30" max="35" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -8017,7 +8017,7 @@
         <v>46234</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -8117,7 +8117,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -8205,7 +8205,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -8299,7 +8299,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -8393,7 +8393,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
@@ -8461,7 +8461,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -8555,7 +8555,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -8649,7 +8649,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>1</v>
       </c>
@@ -8660,7 +8660,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
@@ -8673,7 +8673,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>19</v>
       </c>
@@ -8686,7 +8686,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -8727,30 +8727,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A6D4258-8D1D-40C7-BB83-4C4F9F65CC0B}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -8851,7 +8851,7 @@
         <v>45716</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -8942,7 +8942,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -9027,7 +9027,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -9114,7 +9114,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -9201,7 +9201,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -9286,7 +9286,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -9371,7 +9371,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -9382,7 +9382,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -9395,7 +9395,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -9408,7 +9408,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -9421,7 +9421,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -9434,7 +9434,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -9462,29 +9462,29 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F59B1450-F750-4AAF-92F1-86BC63885A84}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="12.81640625" customWidth="1"/>
-    <col min="8" max="9" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="36" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="12.85546875" customWidth="1"/>
+    <col min="8" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="36" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9594,7 +9594,7 @@
         <v>46265</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -9694,7 +9694,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -9784,7 +9784,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -9874,7 +9874,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -9964,7 +9964,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
@@ -10054,7 +10054,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -10144,7 +10144,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -10234,7 +10234,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>1</v>
       </c>
@@ -10245,7 +10245,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
@@ -10258,7 +10258,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>19</v>
       </c>
@@ -10271,7 +10271,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -10311,29 +10311,29 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57075C38-32AC-4EA3-9612-A4A3D80F7093}">
   <dimension ref="A1:AI18"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="12.81640625" customWidth="1"/>
-    <col min="8" max="9" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="12.85546875" customWidth="1"/>
+    <col min="8" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -10440,7 +10440,7 @@
         <v>46295</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -10537,7 +10537,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -10628,7 +10628,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -10719,7 +10719,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -10810,7 +10810,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
@@ -10901,7 +10901,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -10992,7 +10992,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -11083,7 +11083,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>1</v>
       </c>
@@ -11094,7 +11094,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>30</v>
       </c>
@@ -11107,7 +11107,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>29</v>
       </c>
@@ -11120,7 +11120,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>12</v>
       </c>
@@ -11133,7 +11133,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>31</v>
       </c>
@@ -11146,7 +11146,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>19</v>
       </c>
@@ -11159,7 +11159,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -11199,26 +11199,26 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A2B8991-FECB-4DED-BEB7-2ACC94684DF5}">
   <dimension ref="A1:AJ19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="11" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="18" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="20" max="25" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="27" max="32" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="11" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="18" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="25" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="32" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -11328,7 +11328,7 @@
         <v>46326</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -11428,7 +11428,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -11502,7 +11502,7 @@
       <c r="AI3" s="2"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -11584,7 +11584,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>33</v>
       </c>
@@ -11666,7 +11666,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
@@ -11740,7 +11740,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>31</v>
       </c>
@@ -11801,13 +11801,15 @@
       <c r="X7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="Y7" s="6" t="s">
-        <v>24</v>
+      <c r="Y7" s="5" t="s">
+        <v>17</v>
       </c>
       <c r="Z7" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="AA7" s="2"/>
+      <c r="AA7" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="AB7" s="2"/>
       <c r="AC7" s="7"/>
       <c r="AD7" s="7"/>
@@ -11818,7 +11820,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="7"/>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
@@ -11892,7 +11894,7 @@
       <c r="AI8" s="2"/>
       <c r="AJ8" s="7"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -11968,7 +11970,7 @@
       <c r="AI9" s="2"/>
       <c r="AJ9" s="7"/>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>1</v>
       </c>
@@ -11979,7 +11981,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>30</v>
       </c>
@@ -11992,7 +11994,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>29</v>
       </c>
@@ -12005,7 +12007,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
@@ -12018,7 +12020,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>31</v>
       </c>
@@ -12028,10 +12030,10 @@
       </c>
       <c r="C17" s="2">
         <f t="shared" si="1"/>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>19</v>
       </c>
@@ -12044,7 +12046,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -12084,26 +12086,26 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4E8A644-1993-49C0-933B-42395C786DC4}">
   <dimension ref="A1:AI19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="8" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="10" max="14" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="17" max="22" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="24" max="29" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="31" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="22" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="24" max="29" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="31" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -12210,7 +12212,7 @@
         <v>46356</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -12307,7 +12309,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -12356,7 +12358,7 @@
       <c r="AH3" s="7"/>
       <c r="AI3" s="2"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -12405,7 +12407,7 @@
       <c r="AH4" s="7"/>
       <c r="AI4" s="2"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>33</v>
       </c>
@@ -12462,7 +12464,7 @@
       <c r="AH5" s="7"/>
       <c r="AI5" s="2"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
@@ -12515,7 +12517,7 @@
       <c r="AH6" s="7"/>
       <c r="AI6" s="2"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>31</v>
       </c>
@@ -12564,7 +12566,7 @@
       <c r="AH7" s="7"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
@@ -12615,7 +12617,7 @@
       <c r="AH8" s="7"/>
       <c r="AI8" s="2"/>
     </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -12666,7 +12668,7 @@
       <c r="AH9" s="7"/>
       <c r="AI9" s="2"/>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>1</v>
       </c>
@@ -12677,7 +12679,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>30</v>
       </c>
@@ -12690,7 +12692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>29</v>
       </c>
@@ -12703,7 +12705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
@@ -12716,7 +12718,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>31</v>
       </c>
@@ -12729,7 +12731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>19</v>
       </c>
@@ -12742,7 +12744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -12782,27 +12784,27 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73C05419-3E5B-44D5-9A4D-7C953122A519}">
   <dimension ref="A1:AJ19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="13" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="15" max="20" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="22" max="27" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="29" max="34" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="13" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="20" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="22" max="27" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="29" max="34" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -12912,7 +12914,7 @@
         <v>46387</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -13012,7 +13014,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -13062,7 +13064,7 @@
       <c r="AI3" s="2"/>
       <c r="AJ3" s="2"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -13112,7 +13114,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="2"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>33</v>
       </c>
@@ -13168,7 +13170,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="2"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
@@ -13226,7 +13228,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="2"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>31</v>
       </c>
@@ -13276,7 +13278,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
@@ -13332,7 +13334,7 @@
       <c r="AI8" s="2"/>
       <c r="AJ8" s="2"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -13398,7 +13400,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>1</v>
       </c>
@@ -13409,7 +13411,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>30</v>
       </c>
@@ -13422,7 +13424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>29</v>
       </c>
@@ -13435,7 +13437,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
@@ -13448,7 +13450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>31</v>
       </c>
@@ -13461,7 +13463,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>19</v>
       </c>
@@ -13474,7 +13476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -13515,28 +13517,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E625ADA5-2D1E-431C-8817-0E3A7680EE75}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AJ13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -13646,7 +13648,7 @@
         <v>45747</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -13746,7 +13748,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -13836,7 +13838,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -13924,7 +13926,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="13"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -14012,7 +14014,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="13"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -14100,7 +14102,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="13"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -14138,7 +14140,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="14"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>1</v>
       </c>
@@ -14149,7 +14151,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -14162,7 +14164,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -14175,7 +14177,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -14188,7 +14190,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
@@ -14226,29 +14228,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61D25C68-D147-4871-A2A8-2CD748E8464B}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:AI14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -14355,7 +14357,7 @@
         <v>45777</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -14452,7 +14454,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -14543,7 +14545,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -14634,7 +14636,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -14725,7 +14727,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -14816,7 +14818,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -14853,7 +14855,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -14864,7 +14866,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -14877,7 +14879,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -14890,7 +14892,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -14903,7 +14905,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -14941,29 +14943,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460154BA-7A2B-4633-BD09-4305E2926D5D}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:AJ14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.7265625" bestFit="1" customWidth="1"/>
-    <col min="15" max="18" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="20" max="25" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="27" max="32" width="9.7265625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="18" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="25" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="32" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -15073,7 +15075,7 @@
         <v>45808</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -15173,7 +15175,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -15265,7 +15267,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -15357,7 +15359,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -15449,7 +15451,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -15541,7 +15543,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -15578,7 +15580,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -15589,7 +15591,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -15602,7 +15604,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -15615,7 +15617,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -15628,7 +15630,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -15670,15 +15672,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55B0C082-0457-4696-978D-1BE2DD3075D3}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -15785,7 +15787,7 @@
         <v>45838</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -15882,7 +15884,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -15971,7 +15973,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -16060,7 +16062,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -16149,7 +16151,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -16238,7 +16240,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -16275,7 +16277,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>1</v>
       </c>
@@ -16286,7 +16288,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -16299,7 +16301,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -16312,7 +16314,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -16325,7 +16327,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -16365,17 +16367,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6D2793F-73F1-4265-B1CF-8D693D22CC02}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -16485,7 +16487,7 @@
         <v>45869</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -16585,7 +16587,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -16679,7 +16681,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -16773,7 +16775,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -16867,7 +16869,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -16961,7 +16963,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -16998,7 +17000,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -17009,7 +17011,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -17022,7 +17024,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -17035,7 +17037,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -17048,7 +17050,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -17088,18 +17090,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F16C68-A443-46CF-B7FA-2968469C0FB5}">
   <dimension ref="A1:AK15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -17210,7 +17212,7 @@
       </c>
       <c r="AK1" s="1"/>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -17310,7 +17312,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -17400,7 +17402,7 @@
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -17490,7 +17492,7 @@
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -17580,7 +17582,7 @@
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -17670,7 +17672,7 @@
       <c r="AI6" s="7"/>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -17708,7 +17710,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -17719,7 +17721,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -17732,7 +17734,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -17745,7 +17747,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -17758,7 +17760,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -17798,19 +17800,19 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED7CEAED-F464-426C-A766-484A87191C7F}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -17917,7 +17919,7 @@
         <v>45930</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -18014,7 +18016,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -18105,7 +18107,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -18196,7 +18198,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -18287,7 +18289,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -18378,7 +18380,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -18415,7 +18417,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -18426,7 +18428,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -18439,7 +18441,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -18452,7 +18454,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -18465,7 +18467,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
Daily attendance update - 2026-10-20
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC7516A8-4C2E-4CF4-BA69-1DE18B5A0896}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B148D1A-1A9A-4FF1-9107-8A0E7609CA34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="21" activeTab="21" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="21" activeTab="21" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3478" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3481" uniqueCount="34">
   <si>
     <t>Person</t>
   </si>
@@ -1357,31 +1357,31 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27991520-C614-4BFB-ADD8-628FF075C04B}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="9.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -1491,7 +1491,7 @@
         <v>45688</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -1591,7 +1591,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -1685,7 +1685,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -1779,7 +1779,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -1873,7 +1873,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -1967,7 +1967,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -2061,7 +2061,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -2072,7 +2072,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -2085,7 +2085,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -2098,7 +2098,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -2111,7 +2111,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -2124,7 +2124,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -2153,30 +2153,30 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{826FC1B3-53E6-4D35-9223-A0DEC05CDA48}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="19" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="24" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="28" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="12" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="19" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="21" max="24" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="28" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2286,7 +2286,7 @@
         <v>45961</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -2386,7 +2386,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -2480,7 +2480,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -2574,7 +2574,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -2668,7 +2668,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -2762,7 +2762,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -2800,7 +2800,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -2811,7 +2811,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -2824,7 +2824,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -2837,7 +2837,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -2850,7 +2850,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -2890,26 +2890,26 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C42BC0F2-E7C0-48B4-8AB8-C4D08FDA0656}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -3016,7 +3016,7 @@
         <v>45991</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3113,7 +3113,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -3200,7 +3200,7 @@
       <c r="AH3" s="7"/>
       <c r="AI3" s="7"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -3287,7 +3287,7 @@
       <c r="AH4" s="7"/>
       <c r="AI4" s="7"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -3374,7 +3374,7 @@
       <c r="AH5" s="7"/>
       <c r="AI5" s="7"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -3461,7 +3461,7 @@
       <c r="AH6" s="7"/>
       <c r="AI6" s="7"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -3498,7 +3498,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -3509,7 +3509,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -3522,7 +3522,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -3535,7 +3535,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -3548,7 +3548,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -3588,27 +3588,27 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{988C623D-E1BD-4FE8-8DE5-A86BDEB0A522}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -3718,7 +3718,7 @@
         <v>46022</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -3818,7 +3818,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -3912,7 +3912,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -4006,7 +4006,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4100,7 +4100,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -4194,7 +4194,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -4232,7 +4232,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -4243,7 +4243,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -4256,7 +4256,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -4269,7 +4269,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -4282,7 +4282,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -4322,27 +4322,27 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9E71A27-DC0F-4421-B295-A887695B49EA}">
   <dimension ref="A1:AJ13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -4452,7 +4452,7 @@
         <v>46053</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -4552,7 +4552,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -4644,7 +4644,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -4736,7 +4736,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -4828,7 +4828,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -4866,7 +4866,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="2"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
         <v>1</v>
       </c>
@@ -4877,7 +4877,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -4890,7 +4890,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -4903,7 +4903,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -4943,26 +4943,26 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F94C369-A483-4243-8B30-4AC8F8C2C920}">
   <dimension ref="A1:AG12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -5063,7 +5063,7 @@
         <v>46081</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -5154,7 +5154,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5239,7 +5239,7 @@
       </c>
       <c r="AG3" s="7"/>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5324,7 +5324,7 @@
       </c>
       <c r="AG4" s="7"/>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5409,7 +5409,7 @@
       </c>
       <c r="AG5" s="7"/>
     </row>
-    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>1</v>
       </c>
@@ -5420,7 +5420,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -5433,7 +5433,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -5446,7 +5446,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -5486,27 +5486,27 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72154BF-0805-461D-B9A5-E64EDBF4FEB9}">
   <dimension ref="A1:AJ12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -5616,7 +5616,7 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -5716,7 +5716,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -5808,7 +5808,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -5900,7 +5900,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -5992,7 +5992,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>1</v>
       </c>
@@ -6003,7 +6003,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -6016,7 +6016,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -6029,7 +6029,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -6069,27 +6069,27 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF130E33-32AF-452B-AEB5-3A35260DB102}">
   <dimension ref="A1:AI12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="34" max="35" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="34" max="35" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6196,7 +6196,7 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -6293,7 +6293,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -6384,7 +6384,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -6475,7 +6475,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -6566,7 +6566,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>1</v>
       </c>
@@ -6577,7 +6577,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -6590,7 +6590,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -6603,7 +6603,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -6643,29 +6643,29 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97DA7DA3-001B-413F-BA22-DC9827945C1D}">
   <dimension ref="A1:AJ12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="19" max="24" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="26" max="31" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="33" max="36" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="17" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="19" max="24" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="26" max="31" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="33" max="36" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -6775,7 +6775,7 @@
         <v>46173</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -6875,7 +6875,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -6965,7 +6965,7 @@
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -7055,7 +7055,7 @@
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -7145,7 +7145,7 @@
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
         <v>1</v>
       </c>
@@ -7156,7 +7156,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -7169,7 +7169,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -7182,7 +7182,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -7222,27 +7222,27 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{934EE78C-1B04-4E2F-8C73-18B0A1ECFFAE}">
   <dimension ref="A1:AI13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="21" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="23" max="28" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="30" max="35" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="21" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="23" max="28" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="30" max="35" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -7349,7 +7349,7 @@
         <v>46203</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -7446,7 +7446,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>29</v>
       </c>
@@ -7537,7 +7537,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -7628,7 +7628,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
@@ -7719,7 +7719,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -7810,7 +7810,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
         <v>1</v>
       </c>
@@ -7821,7 +7821,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -7834,7 +7834,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -7847,7 +7847,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -7887,27 +7887,27 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77C449D2-15A1-404E-9EF3-800FA95F32E2}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="21" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="23" max="28" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="30" max="35" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="21" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="23" max="28" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="30" max="35" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -8017,7 +8017,7 @@
         <v>46234</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -8117,7 +8117,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -8205,7 +8205,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -8299,7 +8299,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -8393,7 +8393,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
@@ -8461,7 +8461,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -8555,7 +8555,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -8649,7 +8649,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
         <v>1</v>
       </c>
@@ -8660,7 +8660,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
@@ -8673,7 +8673,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>19</v>
       </c>
@@ -8686,7 +8686,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -8727,30 +8727,30 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A6D4258-8D1D-40C7-BB83-4C4F9F65CC0B}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AG15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="33" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -8851,7 +8851,7 @@
         <v>45716</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -8942,7 +8942,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -9027,7 +9027,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -9114,7 +9114,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -9201,7 +9201,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -9286,7 +9286,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -9371,7 +9371,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -9382,7 +9382,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -9395,7 +9395,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -9408,7 +9408,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -9421,7 +9421,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -9434,7 +9434,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -9462,29 +9462,29 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F59B1450-F750-4AAF-92F1-86BC63885A84}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="12.85546875" customWidth="1"/>
-    <col min="8" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="36" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="12.81640625" customWidth="1"/>
+    <col min="8" max="9" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="36" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9594,7 +9594,7 @@
         <v>46265</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -9694,7 +9694,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -9784,7 +9784,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -9874,7 +9874,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -9964,7 +9964,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
@@ -10054,7 +10054,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -10144,7 +10144,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -10234,7 +10234,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
         <v>1</v>
       </c>
@@ -10245,7 +10245,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
@@ -10258,7 +10258,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>19</v>
       </c>
@@ -10271,7 +10271,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
@@ -10311,29 +10311,29 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57075C38-32AC-4EA3-9612-A4A3D80F7093}">
   <dimension ref="A1:AI18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="12.85546875" customWidth="1"/>
-    <col min="8" max="9" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="23" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="30" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="32" max="35" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="12.81640625" customWidth="1"/>
+    <col min="8" max="9" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="23" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="30" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="35" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -10440,7 +10440,7 @@
         <v>46295</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -10537,7 +10537,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -10628,7 +10628,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -10719,7 +10719,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -10810,7 +10810,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>31</v>
       </c>
@@ -10901,7 +10901,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -10992,7 +10992,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
@@ -11083,7 +11083,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
         <v>1</v>
       </c>
@@ -11094,7 +11094,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>30</v>
       </c>
@@ -11107,7 +11107,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>29</v>
       </c>
@@ -11120,7 +11120,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>12</v>
       </c>
@@ -11133,7 +11133,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>31</v>
       </c>
@@ -11146,7 +11146,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>19</v>
       </c>
@@ -11159,7 +11159,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>20</v>
       </c>
@@ -11199,26 +11199,26 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A2B8991-FECB-4DED-BEB7-2ACC94684DF5}">
   <dimension ref="A1:AJ19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="11" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="18" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="25" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="27" max="32" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="11" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="18" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="20" max="25" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="27" max="32" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -11328,7 +11328,7 @@
         <v>46326</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -11428,7 +11428,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -11502,7 +11502,7 @@
       <c r="AI3" s="2"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -11584,7 +11584,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>33</v>
       </c>
@@ -11666,7 +11666,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
@@ -11744,7 +11744,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>31</v>
       </c>
@@ -11824,7 +11824,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="7"/>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
@@ -11898,7 +11898,7 @@
       <c r="AI8" s="2"/>
       <c r="AJ8" s="7"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -11974,7 +11974,7 @@
       <c r="AI9" s="2"/>
       <c r="AJ9" s="7"/>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
         <v>1</v>
       </c>
@@ -11985,7 +11985,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>30</v>
       </c>
@@ -11998,7 +11998,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>29</v>
       </c>
@@ -12011,7 +12011,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
@@ -12024,7 +12024,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>31</v>
       </c>
@@ -12037,7 +12037,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>19</v>
       </c>
@@ -12050,7 +12050,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -12090,26 +12090,26 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4E8A644-1993-49C0-933B-42395C786DC4}">
   <dimension ref="A1:AI19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="8" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="14" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="22" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="24" max="29" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="31" max="35" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="8" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="14" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="17" max="22" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="24" max="29" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="31" max="35" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -12216,7 +12216,7 @@
         <v>46356</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -12313,7 +12313,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -12362,7 +12362,7 @@
       <c r="AH3" s="7"/>
       <c r="AI3" s="2"/>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -12411,7 +12411,7 @@
       <c r="AH4" s="7"/>
       <c r="AI4" s="2"/>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>33</v>
       </c>
@@ -12468,7 +12468,7 @@
       <c r="AH5" s="7"/>
       <c r="AI5" s="2"/>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
@@ -12521,7 +12521,7 @@
       <c r="AH6" s="7"/>
       <c r="AI6" s="2"/>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>31</v>
       </c>
@@ -12570,7 +12570,7 @@
       <c r="AH7" s="7"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
@@ -12621,7 +12621,7 @@
       <c r="AH8" s="7"/>
       <c r="AI8" s="2"/>
     </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -12672,7 +12672,7 @@
       <c r="AH9" s="7"/>
       <c r="AI9" s="2"/>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
         <v>1</v>
       </c>
@@ -12683,7 +12683,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>30</v>
       </c>
@@ -12696,7 +12696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>29</v>
       </c>
@@ -12709,7 +12709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
@@ -12722,7 +12722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>31</v>
       </c>
@@ -12735,7 +12735,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>19</v>
       </c>
@@ -12748,7 +12748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -12788,27 +12788,27 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73C05419-3E5B-44D5-9A4D-7C953122A519}">
   <dimension ref="A1:AJ19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="13" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="20" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="22" max="27" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="29" max="34" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="13" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="15" max="20" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="22" max="27" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="29" max="34" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="10.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -12918,7 +12918,7 @@
         <v>46387</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -13018,7 +13018,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
@@ -13080,7 +13080,7 @@
       <c r="AI3" s="2"/>
       <c r="AJ3" s="2"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>29</v>
       </c>
@@ -13130,7 +13130,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="2"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>33</v>
       </c>
@@ -13186,7 +13186,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="2"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
@@ -13216,7 +13216,9 @@
       </c>
       <c r="J6" s="7"/>
       <c r="K6" s="7"/>
-      <c r="L6" s="2"/>
+      <c r="L6" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
@@ -13244,7 +13246,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="2"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>31</v>
       </c>
@@ -13294,7 +13296,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
@@ -13327,7 +13329,9 @@
       <c r="T8" s="2"/>
       <c r="U8" s="2"/>
       <c r="V8" s="2"/>
-      <c r="W8" s="2"/>
+      <c r="W8" s="6" t="s">
+        <v>24</v>
+      </c>
       <c r="X8" s="7"/>
       <c r="Y8" s="7"/>
       <c r="Z8" s="2"/>
@@ -13348,9 +13352,11 @@
       </c>
       <c r="AH8" s="2"/>
       <c r="AI8" s="2"/>
-      <c r="AJ8" s="2"/>
-    </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="AJ8" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -13416,7 +13422,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
         <v>1</v>
       </c>
@@ -13427,7 +13433,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>30</v>
       </c>
@@ -13440,7 +13446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>29</v>
       </c>
@@ -13453,7 +13459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>12</v>
       </c>
@@ -13466,7 +13472,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>31</v>
       </c>
@@ -13479,7 +13485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>19</v>
       </c>
@@ -13492,7 +13498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>20</v>
       </c>
@@ -13533,28 +13539,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E625ADA5-2D1E-431C-8817-0E3A7680EE75}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:AJ13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="10.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -13664,7 +13670,7 @@
         <v>45747</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -13764,7 +13770,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -13854,7 +13860,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -13942,7 +13948,7 @@
       <c r="AI4" s="2"/>
       <c r="AJ4" s="13"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -14030,7 +14036,7 @@
       <c r="AI5" s="2"/>
       <c r="AJ5" s="13"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -14118,7 +14124,7 @@
       <c r="AI6" s="2"/>
       <c r="AJ6" s="13"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -14156,7 +14162,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="14"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
         <v>1</v>
       </c>
@@ -14167,7 +14173,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
@@ -14180,7 +14186,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>19</v>
       </c>
@@ -14193,7 +14199,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -14206,7 +14212,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
@@ -14244,29 +14250,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61D25C68-D147-4871-A2A8-2CD748E8464B}">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:AI14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="15" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="18" max="23" width="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="25" max="30" width="10" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="11.26953125" bestFit="1" customWidth="1"/>
     <col min="32" max="35" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -14373,7 +14379,7 @@
         <v>45777</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -14470,7 +14476,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -14561,7 +14567,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -14652,7 +14658,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -14743,7 +14749,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -14834,7 +14840,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -14871,7 +14877,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -14882,7 +14888,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -14895,7 +14901,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -14908,7 +14914,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -14921,7 +14927,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -14959,29 +14965,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{460154BA-7A2B-4633-BD09-4305E2926D5D}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:AJ14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="18" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="20" max="25" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="27" max="32" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="34" max="36" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="15" max="18" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="20" max="25" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="27" max="32" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="34" max="36" width="9.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -15091,7 +15097,7 @@
         <v>45808</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -15191,7 +15197,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -15283,7 +15289,7 @@
       </c>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -15375,7 +15381,7 @@
       </c>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -15467,7 +15473,7 @@
       </c>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -15559,7 +15565,7 @@
       </c>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -15596,7 +15602,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>1</v>
       </c>
@@ -15607,7 +15613,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -15620,7 +15626,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>19</v>
       </c>
@@ -15633,7 +15639,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>20</v>
       </c>
@@ -15646,7 +15652,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>23</v>
       </c>
@@ -15688,15 +15694,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55B0C082-0457-4696-978D-1BE2DD3075D3}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -15803,7 +15809,7 @@
         <v>45838</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -15900,7 +15906,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -15989,7 +15995,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -16078,7 +16084,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -16167,7 +16173,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -16256,7 +16262,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -16293,7 +16299,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
         <v>1</v>
       </c>
@@ -16304,7 +16310,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -16317,7 +16323,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -16330,7 +16336,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -16343,7 +16349,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -16383,17 +16389,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6D2793F-73F1-4265-B1CF-8D693D22CC02}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -16503,7 +16509,7 @@
         <v>45869</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -16603,7 +16609,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -16697,7 +16703,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -16791,7 +16797,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -16885,7 +16891,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -16979,7 +16985,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -17016,7 +17022,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -17027,7 +17033,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -17040,7 +17046,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -17053,7 +17059,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -17066,7 +17072,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -17106,18 +17112,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F16C68-A443-46CF-B7FA-2968469C0FB5}">
   <dimension ref="A1:AK15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -17228,7 +17234,7 @@
       </c>
       <c r="AK1" s="1"/>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -17328,7 +17334,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -17418,7 +17424,7 @@
       <c r="AI3" s="7"/>
       <c r="AJ3" s="7"/>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -17508,7 +17514,7 @@
       <c r="AI4" s="7"/>
       <c r="AJ4" s="7"/>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -17598,7 +17604,7 @@
       <c r="AI5" s="7"/>
       <c r="AJ5" s="7"/>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -17688,7 +17694,7 @@
       <c r="AI6" s="7"/>
       <c r="AJ6" s="7"/>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -17726,7 +17732,7 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -17737,7 +17743,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -17750,7 +17756,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -17763,7 +17769,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -17776,7 +17782,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>
@@ -17816,19 +17822,19 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED7CEAED-F464-426C-A766-484A87191C7F}">
   <dimension ref="A1:AI15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -17935,7 +17941,7 @@
         <v>45930</v>
       </c>
     </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" s="11"/>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -18032,7 +18038,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -18123,7 +18129,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -18214,7 +18220,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -18305,7 +18311,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>23</v>
       </c>
@@ -18396,7 +18402,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -18433,7 +18439,7 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
     </row>
-    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
         <v>1</v>
       </c>
@@ -18444,7 +18450,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -18457,7 +18463,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>19</v>
       </c>
@@ -18470,7 +18476,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>20</v>
       </c>
@@ -18483,7 +18489,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
Daily attendance update - 2026-10-22
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2352DF9D-FAC7-41D2-B2A7-657DC382A83D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6499892D-80DB-4A92-8B80-74C9E856FE70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="21" activeTab="23" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="21" activeTab="21" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3491" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3503" uniqueCount="34">
   <si>
     <t>Person</t>
   </si>
@@ -11492,9 +11492,15 @@
       <c r="Y3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="Z3" s="2"/>
-      <c r="AA3" s="2"/>
-      <c r="AB3" s="2"/>
+      <c r="Z3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AA3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB3" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AC3" s="7"/>
       <c r="AD3" s="7"/>
       <c r="AE3" s="2"/>
@@ -11737,8 +11743,12 @@
       <c r="Z6" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="AA6" s="2"/>
-      <c r="AB6" s="2"/>
+      <c r="AA6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB6" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AC6" s="7"/>
       <c r="AD6" s="7"/>
       <c r="AE6" s="2"/>
@@ -11818,7 +11828,9 @@
       <c r="AA7" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="AB7" s="2"/>
+      <c r="AB7" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AC7" s="7"/>
       <c r="AD7" s="7"/>
       <c r="AE7" s="2"/>
@@ -11892,9 +11904,15 @@
       <c r="Y8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="Z8" s="2"/>
-      <c r="AA8" s="2"/>
-      <c r="AB8" s="2"/>
+      <c r="Z8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AA8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AB8" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AC8" s="7"/>
       <c r="AD8" s="7"/>
       <c r="AE8" s="2"/>
@@ -11968,9 +11986,15 @@
       <c r="Y9" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="Z9" s="2"/>
-      <c r="AA9" s="2"/>
-      <c r="AB9" s="2"/>
+      <c r="Z9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AA9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB9" s="5" t="s">
+        <v>17</v>
+      </c>
       <c r="AC9" s="7"/>
       <c r="AD9" s="7"/>
       <c r="AE9" s="2"/>
@@ -12001,7 +12025,7 @@
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(H3:AI3,"WFH")</f>
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:36" x14ac:dyDescent="0.25">
@@ -12027,7 +12051,7 @@
       </c>
       <c r="C16" s="2">
         <f t="shared" ref="C16:C19" si="1">COUNTIF(H6:AI6,"WFH")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -12040,7 +12064,7 @@
       </c>
       <c r="C17" s="2">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -12049,11 +12073,11 @@
       </c>
       <c r="B18" s="2">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C18" s="2">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -12066,7 +12090,7 @@
       </c>
       <c r="C19" s="2">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily attendance update - 2026-10-26
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6499892D-80DB-4A92-8B80-74C9E856FE70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09802DD0-1DC8-46C4-819B-2467CF6531A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="21" activeTab="21" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="21" activeTab="21" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
   <sheets>
     <sheet name="UV-WMS Admin Jan 2025" sheetId="9" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3503" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3509" uniqueCount="34">
   <si>
     <t>Person</t>
   </si>
@@ -11503,7 +11503,9 @@
       </c>
       <c r="AC3" s="7"/>
       <c r="AD3" s="7"/>
-      <c r="AE3" s="2"/>
+      <c r="AE3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AF3" s="2"/>
       <c r="AG3" s="2"/>
       <c r="AH3" s="2"/>
@@ -11585,7 +11587,9 @@
       </c>
       <c r="AC4" s="7"/>
       <c r="AD4" s="7"/>
-      <c r="AE4" s="2"/>
+      <c r="AE4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AF4" s="2"/>
       <c r="AG4" s="2"/>
       <c r="AH4" s="2"/>
@@ -11751,7 +11755,9 @@
       </c>
       <c r="AC6" s="7"/>
       <c r="AD6" s="7"/>
-      <c r="AE6" s="2"/>
+      <c r="AE6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AF6" s="2"/>
       <c r="AG6" s="2"/>
       <c r="AH6" s="2"/>
@@ -11833,7 +11839,9 @@
       </c>
       <c r="AC7" s="7"/>
       <c r="AD7" s="7"/>
-      <c r="AE7" s="2"/>
+      <c r="AE7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AF7" s="2"/>
       <c r="AG7" s="2"/>
       <c r="AH7" s="2"/>
@@ -11915,7 +11923,9 @@
       </c>
       <c r="AC8" s="7"/>
       <c r="AD8" s="7"/>
-      <c r="AE8" s="2"/>
+      <c r="AE8" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AF8" s="2"/>
       <c r="AG8" s="2"/>
       <c r="AH8" s="2"/>
@@ -11997,7 +12007,9 @@
       </c>
       <c r="AC9" s="7"/>
       <c r="AD9" s="7"/>
-      <c r="AE9" s="2"/>
+      <c r="AE9" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AF9" s="2"/>
       <c r="AG9" s="2"/>
       <c r="AH9" s="2"/>
@@ -12021,7 +12033,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(H3:AI3,"WFH")</f>
@@ -12034,7 +12046,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(H4:AI4,"WFH")</f>
@@ -12047,7 +12059,7 @@
       </c>
       <c r="B16" s="2">
         <f t="shared" ref="B16:B19" si="0">COUNTIF(F6:AI6,"WFO")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C16" s="2">
         <f t="shared" ref="C16:C19" si="1">COUNTIF(H6:AI6,"WFH")</f>
@@ -12060,7 +12072,7 @@
       </c>
       <c r="B17" s="2">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C17" s="2">
         <f t="shared" si="1"/>
@@ -12073,7 +12085,7 @@
       </c>
       <c r="B18" s="2">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C18" s="2">
         <f t="shared" si="1"/>
@@ -12086,7 +12098,7 @@
       </c>
       <c r="B19" s="2">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C19" s="2">
         <f t="shared" si="1"/>

</xml_diff>

<commit_message>
Daily attendance update - 2026-10-28
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09802DD0-1DC8-46C4-819B-2467CF6531A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A21B24-B6AC-4054-8E35-30C66A661857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="21" activeTab="21" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3509" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3523" uniqueCount="34">
   <si>
     <t>Person</t>
   </si>
@@ -11506,8 +11506,12 @@
       <c r="AE3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AF3" s="2"/>
-      <c r="AG3" s="2"/>
+      <c r="AF3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AH3" s="2"/>
       <c r="AI3" s="2"/>
       <c r="AJ3" s="7"/>
@@ -11590,8 +11594,12 @@
       <c r="AE4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AF4" s="2"/>
-      <c r="AG4" s="2"/>
+      <c r="AF4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG4" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AH4" s="2"/>
       <c r="AI4" s="2"/>
       <c r="AJ4" s="7"/>
@@ -11674,8 +11682,12 @@
       <c r="AE5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="AF5" s="2"/>
-      <c r="AG5" s="2"/>
+      <c r="AF5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AH5" s="2"/>
       <c r="AI5" s="2"/>
       <c r="AJ5" s="7"/>
@@ -11758,8 +11770,12 @@
       <c r="AE6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AF6" s="2"/>
-      <c r="AG6" s="2"/>
+      <c r="AF6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AH6" s="2"/>
       <c r="AI6" s="2"/>
       <c r="AJ6" s="7"/>
@@ -11842,8 +11858,12 @@
       <c r="AE7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AF7" s="2"/>
-      <c r="AG7" s="2"/>
+      <c r="AF7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
       <c r="AJ7" s="7"/>
@@ -11926,8 +11946,12 @@
       <c r="AE8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AF8" s="2"/>
-      <c r="AG8" s="2"/>
+      <c r="AF8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG8" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AH8" s="2"/>
       <c r="AI8" s="2"/>
       <c r="AJ8" s="7"/>
@@ -12010,8 +12034,12 @@
       <c r="AE9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AF9" s="2"/>
-      <c r="AG9" s="2"/>
+      <c r="AF9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="AG9" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AH9" s="2"/>
       <c r="AI9" s="2"/>
       <c r="AJ9" s="7"/>
@@ -12033,7 +12061,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(H3:AI3,"WFH")</f>
@@ -12046,7 +12074,7 @@
       </c>
       <c r="B15" s="2">
         <f>COUNTIF(F4:AI4,"WFO")</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C15" s="2">
         <f>COUNTIF(H4:AI4,"WFH")</f>
@@ -12059,7 +12087,7 @@
       </c>
       <c r="B16" s="2">
         <f t="shared" ref="B16:B19" si="0">COUNTIF(F6:AI6,"WFO")</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C16" s="2">
         <f t="shared" ref="C16:C19" si="1">COUNTIF(H6:AI6,"WFH")</f>
@@ -12072,7 +12100,7 @@
       </c>
       <c r="B17" s="2">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C17" s="2">
         <f t="shared" si="1"/>
@@ -12085,7 +12113,7 @@
       </c>
       <c r="B18" s="2">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C18" s="2">
         <f t="shared" si="1"/>
@@ -12098,7 +12126,7 @@
       </c>
       <c r="B19" s="2">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C19" s="2">
         <f t="shared" si="1"/>

</xml_diff>

<commit_message>
Daily attendance update - 2026-10-29
</commit_message>
<xml_diff>
--- a/data/App_Admin_UV-WCS.xlsx
+++ b/data/App_Admin_UV-WCS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\rethin\projects\wfo_tracker\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7A21B24-B6AC-4054-8E35-30C66A661857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17493E7A-74F2-4183-A46A-3F5E39FFA5D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="21" activeTab="21" xr2:uid="{BB3BFA0C-538F-411B-ABFF-D727D65D2D40}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3523" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3530" uniqueCount="34">
   <si>
     <t>Person</t>
   </si>
@@ -11512,7 +11512,9 @@
       <c r="AG3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AH3" s="2"/>
+      <c r="AH3" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AI3" s="2"/>
       <c r="AJ3" s="7"/>
     </row>
@@ -11600,7 +11602,9 @@
       <c r="AG4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AH4" s="2"/>
+      <c r="AH4" s="6" t="s">
+        <v>18</v>
+      </c>
       <c r="AI4" s="2"/>
       <c r="AJ4" s="7"/>
     </row>
@@ -11688,7 +11692,9 @@
       <c r="AG5" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AH5" s="2"/>
+      <c r="AH5" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AI5" s="2"/>
       <c r="AJ5" s="7"/>
     </row>
@@ -11776,7 +11782,9 @@
       <c r="AG6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AH6" s="2"/>
+      <c r="AH6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AI6" s="2"/>
       <c r="AJ6" s="7"/>
     </row>
@@ -11864,7 +11872,9 @@
       <c r="AG7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AH7" s="2"/>
+      <c r="AH7" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AI7" s="2"/>
       <c r="AJ7" s="7"/>
     </row>
@@ -11952,7 +11962,9 @@
       <c r="AG8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AH8" s="2"/>
+      <c r="AH8" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AI8" s="2"/>
       <c r="AJ8" s="7"/>
     </row>
@@ -12040,7 +12052,9 @@
       <c r="AG9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="AH9" s="2"/>
+      <c r="AH9" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="AI9" s="2"/>
       <c r="AJ9" s="7"/>
     </row>
@@ -12061,7 +12075,7 @@
       </c>
       <c r="B14" s="2">
         <f>COUNTIF(F3:AI3,"WFO")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C14" s="2">
         <f>COUNTIF(H3:AI3,"WFH")</f>
@@ -12087,7 +12101,7 @@
       </c>
       <c r="B16" s="2">
         <f t="shared" ref="B16:B19" si="0">COUNTIF(F6:AI6,"WFO")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C16" s="2">
         <f t="shared" ref="C16:C19" si="1">COUNTIF(H6:AI6,"WFH")</f>
@@ -12100,7 +12114,7 @@
       </c>
       <c r="B17" s="2">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C17" s="2">
         <f t="shared" si="1"/>
@@ -12113,7 +12127,7 @@
       </c>
       <c r="B18" s="2">
         <f t="shared" si="0"/>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C18" s="2">
         <f t="shared" si="1"/>
@@ -12126,7 +12140,7 @@
       </c>
       <c r="B19" s="2">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C19" s="2">
         <f t="shared" si="1"/>

</xml_diff>